<commit_message>
Updated rates to be in 2023 dollars
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97CAFAC6-7951-4B27-8537-36DD98E5D2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A93C891-BDDA-407D-BD69-0AD2A78BCBC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10320" activeTab="2" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="2" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -433,6 +433,7 @@
     <author>tc={30E6622D-E007-41AB-B0B0-A6FA07445B38}</author>
     <author>tc={CC2FED43-9317-4942-84AB-D91CBD6CC0A1}</author>
     <author>tc={964F0726-9326-406D-BF37-7999B0A6D102}</author>
+    <author>tc={936919AF-DC5C-473D-ADF0-F77CA44CF3E1}</author>
   </authors>
   <commentList>
     <comment ref="G2" authorId="0" shapeId="0" xr:uid="{91B01F22-295E-46BB-ACCB-2E4ED162A079}">
@@ -485,6 +486,14 @@
     Calculated by manually adding in the cost of startup</t>
       </text>
     </comment>
+    <comment ref="A15" authorId="6" shapeId="0" xr:uid="{936919AF-DC5C-473D-ADF0-F77CA44CF3E1}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    These are now all incorrect with the updated RTP rate</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -810,7 +819,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -977,6 +986,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="35">
@@ -1943,28 +1958,31 @@
   <threadedComment ref="O13" dT="2026-08-31T20:52:23.61" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{964F0726-9326-406D-BF37-7999B0A6D102}">
     <text>Calculated by manually adding in the cost of startup</text>
   </threadedComment>
+  <threadedComment ref="A15" dT="2026-09-11T20:08:59.21" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{936919AF-DC5C-473D-ADF0-F77CA44CF3E1}">
+    <text>These are now all incorrect with the updated RTP rate</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
   <dimension ref="A1:V123"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.61328125" customWidth="1"/>
-    <col min="3" max="3" width="10.84375" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" customWidth="1"/>
+    <col min="3" max="3" width="10.81640625" customWidth="1"/>
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.23046875" customWidth="1"/>
-    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.69140625" customWidth="1"/>
-    <col min="9" max="9" width="9.07421875" customWidth="1"/>
-    <col min="11" max="11" width="10.84375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.53515625" customWidth="1"/>
-    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.84375" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7265625" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" customWidth="1"/>
+    <col min="11" max="11" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.54296875" customWidth="1"/>
+    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1975,7 +1993,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2043,7 +2061,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -2107,7 +2125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -2171,14 +2189,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G5" s="4"/>
       <c r="K5" s="10">
         <f>K4+L4+M4</f>
         <v>85444.512881154791</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -2242,7 +2260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -2306,10 +2324,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -2373,7 +2391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2437,10 +2455,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -2504,7 +2522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -2568,10 +2586,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2633,7 +2651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2689,10 +2707,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2756,7 +2774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2820,7 +2838,7 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="K20">
@@ -2829,7 +2847,7 @@
       </c>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2840,7 +2858,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2904,10 +2922,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2971,7 +2989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -3041,11 +3059,11 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -3109,7 +3127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -3173,10 +3191,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -3240,7 +3258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -3310,7 +3328,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -3380,7 +3398,7 @@
         <v>277.67302057784298</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A33" s="26" t="s">
         <v>45</v>
       </c>
@@ -3463,19 +3481,19 @@
         <v>200.18128127969257</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="K34" s="10"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -3539,7 +3557,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -3603,12 +3621,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A38" s="7"/>
       <c r="B38" s="2"/>
       <c r="S38" s="2"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>20</v>
       </c>
@@ -3675,7 +3693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>22</v>
       </c>
@@ -3745,20 +3763,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3822,15 +3840,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -3900,13 +3918,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>20</v>
       </c>
@@ -3970,7 +3988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>22</v>
       </c>
@@ -4034,11 +4052,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>20</v>
       </c>
@@ -4102,7 +4120,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -4166,10 +4184,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>20</v>
       </c>
@@ -4233,7 +4251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>22</v>
       </c>
@@ -4303,19 +4321,19 @@
         <v>358.72983861659498</v>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
       <c r="K58">
         <f>K57+L57+M57-K5</f>
         <v>5401.088917483823</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>22</v>
       </c>
@@ -4379,7 +4397,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
         <v>22</v>
       </c>
@@ -4444,7 +4462,7 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
         <v>22</v>
       </c>
@@ -4514,7 +4532,7 @@
         <v>278.17977348178903</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -4584,7 +4602,7 @@
         <v>107.018147807505</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A64" s="26" t="s">
         <v>44</v>
       </c>
@@ -4667,19 +4685,19 @@
         <v>-171.16162567428404</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A66" s="9"/>
       <c r="B66" s="9"/>
       <c r="C66" s="9"/>
       <c r="D66" s="13"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A67" s="26" t="s">
         <v>60</v>
       </c>
@@ -4687,7 +4705,7 @@
       <c r="C67" s="26"/>
       <c r="D67" s="10"/>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
         <v>22</v>
       </c>
@@ -4757,7 +4775,7 @@
         <v>350.36946039055402</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A69" s="26" t="s">
         <v>61</v>
       </c>
@@ -4816,7 +4834,7 @@
         <v>133.12347700700047</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A70" s="9"/>
       <c r="B70" s="9"/>
       <c r="C70" s="9"/>
@@ -4837,13 +4855,13 @@
       <c r="O70" s="10"/>
       <c r="P70" s="10"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G71" s="4"/>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -4855,7 +4873,7 @@
       </c>
       <c r="G72" s="4"/>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>22</v>
       </c>
@@ -4919,13 +4937,13 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
       <c r="G74" s="4"/>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
         <v>20</v>
       </c>
@@ -4937,7 +4955,7 @@
       </c>
       <c r="G75" s="4"/>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>22</v>
       </c>
@@ -5006,7 +5024,7 @@
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="D77">
@@ -5086,12 +5104,12 @@
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A79" s="3" t="s">
         <v>20</v>
       </c>
@@ -5155,7 +5173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A80" s="3" t="s">
         <v>22</v>
       </c>
@@ -5219,10 +5237,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A81" s="1"/>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>20</v>
       </c>
@@ -5280,7 +5298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>22</v>
       </c>
@@ -5344,7 +5362,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>20</v>
       </c>
@@ -5402,7 +5420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>22</v>
       </c>
@@ -5472,7 +5490,7 @@
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.35">
       <c r="D87">
         <f>D86-D80</f>
         <v>-4018.7603482047853</v>
@@ -5522,13 +5540,13 @@
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G88" s="4"/>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>22</v>
       </c>
@@ -5592,7 +5610,7 @@
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>22</v>
       </c>
@@ -5636,8 +5654,8 @@
         <v>36</v>
       </c>
     </row>
-    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.4"/>
-    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>26</v>
       </c>
@@ -5658,7 +5676,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>0</v>
       </c>
@@ -5720,10 +5738,10 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G94" s="4"/>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>20</v>
       </c>
@@ -5793,7 +5811,7 @@
         <v>319.37310450388202</v>
       </c>
     </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A96" s="3" t="s">
         <v>20</v>
       </c>
@@ -5838,16 +5856,16 @@
         <v>36</v>
       </c>
     </row>
-    <row r="97" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A97" s="2"/>
       <c r="G97" s="4"/>
     </row>
-    <row r="99" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>22</v>
       </c>
@@ -5900,7 +5918,7 @@
         <v>265201.24508552696</v>
       </c>
     </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>22</v>
       </c>
@@ -5970,13 +5988,13 @@
         <v>290.07670650869801</v>
       </c>
     </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="102" spans="1:22" x14ac:dyDescent="0.35">
       <c r="K102">
         <f>SUM(K100:M100)-SUM(K101:M101)</f>
         <v>-750.09243586547382</v>
       </c>
     </row>
-    <row r="103" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>22</v>
       </c>
@@ -6026,7 +6044,7 @@
         <v>303282.7899059637</v>
       </c>
     </row>
-    <row r="104" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>22</v>
       </c>
@@ -6096,19 +6114,19 @@
         <v>351.71871156820202</v>
       </c>
     </row>
-    <row r="105" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="105" spans="1:22" x14ac:dyDescent="0.35">
       <c r="K105" s="13">
         <f>SUM(K103:M103)-SUM(K104:M104)</f>
         <v>-831.26776848098962</v>
       </c>
     </row>
-    <row r="106" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="106" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>65</v>
       </c>
       <c r="K106" s="13"/>
     </row>
-    <row r="107" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="107" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>22</v>
       </c>
@@ -6178,7 +6196,7 @@
         <v>359.195907759661</v>
       </c>
     </row>
-    <row r="108" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>22</v>
       </c>
@@ -6248,7 +6266,7 @@
         <v>331.01860370537798</v>
       </c>
     </row>
-    <row r="109" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="109" spans="1:22" x14ac:dyDescent="0.35">
       <c r="D109" s="13">
         <f>D108-D31</f>
         <v>870.81314264753019</v>
@@ -6294,7 +6312,7 @@
         <v>-2.9942133752499558</v>
       </c>
     </row>
-    <row r="110" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="110" spans="1:22" x14ac:dyDescent="0.35">
       <c r="D110" s="13"/>
       <c r="E110" s="13"/>
       <c r="F110" s="13"/>
@@ -6307,7 +6325,7 @@
       <c r="M110" s="13"/>
       <c r="N110" s="13"/>
     </row>
-    <row r="111" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="111" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>66</v>
       </c>
@@ -6323,7 +6341,7 @@
       <c r="M111" s="13"/>
       <c r="N111" s="13"/>
     </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="112" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>22</v>
       </c>
@@ -6393,7 +6411,7 @@
         <v>300.72865279776499</v>
       </c>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.35">
       <c r="D113" s="12">
         <f>(D112-D4)</f>
         <v>-7531.9083775022591</v>
@@ -6409,7 +6427,7 @@
       <c r="M113" s="13"/>
       <c r="N113" s="13"/>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.35">
       <c r="D114" s="13"/>
       <c r="E114" s="13"/>
       <c r="F114" s="13"/>
@@ -6422,12 +6440,12 @@
       <c r="M114" s="13"/>
       <c r="N114" s="13"/>
     </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="115" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A115" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>32</v>
       </c>
@@ -6438,7 +6456,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>20</v>
       </c>
@@ -6502,7 +6520,7 @@
         <v>0.12591688076390301</v>
       </c>
     </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>20</v>
       </c>
@@ -6566,7 +6584,7 @@
         <v>0.14758705239613301</v>
       </c>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="119" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>20</v>
       </c>
@@ -6630,7 +6648,7 @@
         <v>-0.25983751983286502</v>
       </c>
     </row>
-    <row r="120" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="120" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>20</v>
       </c>
@@ -6694,7 +6712,7 @@
         <v>0.28049716262959101</v>
       </c>
     </row>
-    <row r="121" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="121" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A121" s="3">
         <v>20</v>
       </c>
@@ -6758,7 +6776,7 @@
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="122" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>20</v>
       </c>
@@ -6822,7 +6840,7 @@
         <v>0.46004655114715598</v>
       </c>
     </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="123" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>20</v>
       </c>
@@ -6902,20 +6920,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA993591-8C1F-4C7B-A75D-E9726DFB461B}">
   <dimension ref="A2:P31"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="12.84375" customWidth="1"/>
-    <col min="3" max="3" width="11.3828125" customWidth="1"/>
-    <col min="4" max="4" width="15.53515625" customWidth="1"/>
+    <col min="2" max="2" width="12.81640625" customWidth="1"/>
+    <col min="3" max="3" width="11.36328125" customWidth="1"/>
+    <col min="4" max="4" width="15.54296875" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="17.07421875" customWidth="1"/>
-    <col min="7" max="7" width="15.23046875" customWidth="1"/>
-    <col min="8" max="8" width="13.23046875" customWidth="1"/>
-    <col min="9" max="11" width="11.3828125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" customWidth="1"/>
+    <col min="7" max="7" width="15.26953125" customWidth="1"/>
+    <col min="8" max="8" width="13.26953125" customWidth="1"/>
+    <col min="9" max="11" width="11.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -6954,12 +6972,12 @@
       </c>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -6998,7 +7016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="D5" s="10"/>
@@ -7010,7 +7028,7 @@
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>48</v>
       </c>
@@ -7027,7 +7045,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -7067,7 +7085,7 @@
       </c>
       <c r="M7" s="11"/>
     </row>
-    <row r="8" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D8" s="10">
         <f t="shared" ref="D8:K8" si="0">D7-D4</f>
         <v>759.28494035729091</v>
@@ -7102,7 +7120,7 @@
       </c>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>62</v>
       </c>
@@ -7116,7 +7134,7 @@
       <c r="K9" s="10"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>21</v>
       </c>
@@ -7152,7 +7170,7 @@
       </c>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="D11">
         <f>(34653-H10-I11+wrd_pricetater_flex_type_summar!K5+L10)/34653</f>
         <v>0.17154119896168271</v>
@@ -7169,7 +7187,7 @@
       <c r="K11" s="10"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>49</v>
       </c>
@@ -7183,7 +7201,7 @@
       <c r="K12" s="10"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>22</v>
       </c>
@@ -7223,7 +7241,7 @@
       </c>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="D14" s="10"/>
@@ -7236,7 +7254,7 @@
       <c r="K14" s="10"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>46</v>
       </c>
@@ -7249,7 +7267,7 @@
       <c r="J15" s="10"/>
       <c r="K15" s="10"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -7288,7 +7306,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
       <c r="D17">
         <f>(34653-H16-I17+wrd_pricetater_flex_type_summar!K5+L16)/34653</f>
         <v>0.38932217950875497</v>
@@ -7298,7 +7316,7 @@
         <v>87792.098602195503</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>57</v>
       </c>
@@ -7337,7 +7355,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -7345,7 +7363,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>52</v>
       </c>
@@ -7383,7 +7401,7 @@
       </c>
       <c r="L23" s="10"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>55</v>
       </c>
@@ -7421,7 +7439,7 @@
       </c>
       <c r="L25" s="10"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -7458,7 +7476,7 @@
         <v>-476.58002357000078</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -7495,7 +7513,7 @@
         <v>174.37684745549996</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>58</v>
       </c>
@@ -7541,25 +7559,25 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BC34AED-31C3-47D6-9398-9693457BF528}">
   <dimension ref="A1:AB19"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.921875" customWidth="1"/>
-    <col min="2" max="2" width="14.69140625" customWidth="1"/>
-    <col min="3" max="3" width="12.07421875" customWidth="1"/>
+    <col min="1" max="1" width="26.90625" customWidth="1"/>
+    <col min="2" max="2" width="14.7265625" customWidth="1"/>
+    <col min="3" max="3" width="12.08984375" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="8.53515625" customWidth="1"/>
-    <col min="6" max="6" width="11.3828125" customWidth="1"/>
-    <col min="7" max="7" width="15.07421875" customWidth="1"/>
-    <col min="8" max="8" width="10.15234375" customWidth="1"/>
-    <col min="9" max="9" width="11.3828125" customWidth="1"/>
+    <col min="5" max="5" width="8.54296875" customWidth="1"/>
+    <col min="6" max="6" width="11.36328125" customWidth="1"/>
+    <col min="7" max="7" width="15.08984375" customWidth="1"/>
+    <col min="8" max="8" width="10.1796875" customWidth="1"/>
+    <col min="9" max="9" width="11.36328125" customWidth="1"/>
     <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.921875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.69140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="10.69140625" customWidth="1"/>
-    <col min="28" max="28" width="13.84375" customWidth="1"/>
+    <col min="11" max="11" width="16.90625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.7265625" customWidth="1"/>
+    <col min="28" max="28" width="13.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
       <c r="G1">
         <v>121507.92454383519</v>
       </c>
@@ -7567,7 +7585,7 @@
         <v>34653.411662680403</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>67</v>
       </c>
@@ -7653,7 +7671,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>0</v>
       </c>
@@ -7743,7 +7761,7 @@
         <v>0.21734969274652002</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>0.215</v>
       </c>
@@ -7833,7 +7851,7 @@
         <v>0.14991564378830438</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>0.43</v>
       </c>
@@ -7924,7 +7942,7 @@
         <v>0.1072768553096176</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>0.86</v>
       </c>
@@ -8015,7 +8033,7 @@
         <v>0.1072768553096176</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1.29</v>
       </c>
@@ -8106,14 +8124,14 @@
         <v>0.1072768553096176</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="21" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:28" s="21" customFormat="1" x14ac:dyDescent="0.35">
       <c r="D8" s="22"/>
       <c r="E8" s="22"/>
       <c r="Q8" s="23"/>
       <c r="AA8" s="24"/>
       <c r="AB8" s="25"/>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>0</v>
       </c>
@@ -8220,7 +8238,7 @@
         <v>0.53535589967557295</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>0.215</v>
       </c>
@@ -8327,7 +8345,7 @@
         <v>0.46792185071735731</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>0.43</v>
       </c>
@@ -8418,7 +8436,7 @@
         <v>0.40263355404451467</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>0.86</v>
       </c>
@@ -8508,7 +8526,7 @@
         <v>0.36082050708979968</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1.29</v>
       </c>
@@ -8599,15 +8617,15 @@
         <v>0.33396366478241479</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="21" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:28" s="21" customFormat="1" x14ac:dyDescent="0.35">
       <c r="AA14" s="24"/>
       <c r="AB14" s="25"/>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.4">
-      <c r="A15">
-        <v>0</v>
-      </c>
-      <c r="B15" t="s">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="A15" s="2">
+        <v>0</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>72</v>
       </c>
       <c r="C15">
@@ -8693,11 +8711,11 @@
         <v>0.67280721058037529</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.4">
-      <c r="A16">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="A16" s="2">
         <v>0.215</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>72</v>
       </c>
       <c r="C16">
@@ -8783,11 +8801,11 @@
         <v>0.64784363750995022</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.4">
-      <c r="A17">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="A17" s="2">
         <v>0.43</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>72</v>
       </c>
       <c r="C17">
@@ -8874,11 +8892,11 @@
         <v>0.63256386175391488</v>
       </c>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.4">
-      <c r="A18">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="A18" s="2">
         <v>0.86</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="2" t="s">
         <v>72</v>
       </c>
       <c r="C18">
@@ -8964,11 +8982,11 @@
         <v>0.58579049127122573</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.4">
-      <c r="A19">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="A19" s="2">
         <v>1.29</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="2" t="s">
         <v>72</v>
       </c>
       <c r="C19">
@@ -9064,24 +9082,24 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FD55A87-71DC-49C4-874A-7F05794F4461}">
   <dimension ref="A3:P22"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="12.61328125" customWidth="1"/>
-    <col min="3" max="3" width="9.69140625" customWidth="1"/>
-    <col min="4" max="4" width="12.4609375" customWidth="1"/>
+    <col min="2" max="2" width="12.6328125" customWidth="1"/>
+    <col min="3" max="3" width="9.7265625" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="20.921875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.23046875" customWidth="1"/>
-    <col min="8" max="8" width="18.53515625" customWidth="1"/>
-    <col min="9" max="9" width="20.15234375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.07421875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.3828125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.23046875" customWidth="1"/>
-    <col min="13" max="13" width="9.3828125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.15234375" customWidth="1"/>
+    <col min="6" max="6" width="20.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.26953125" customWidth="1"/>
+    <col min="8" max="8" width="18.54296875" customWidth="1"/>
+    <col min="9" max="9" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.26953125" customWidth="1"/>
+    <col min="13" max="13" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
         <v>76</v>
       </c>
@@ -9104,7 +9122,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>101</v>
       </c>
@@ -9133,7 +9151,7 @@
         <v>-4.0410044714229976</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C5">
         <v>10000</v>
       </c>
@@ -9155,7 +9173,7 @@
         <v>-12815.109372157822</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C6">
         <v>12000</v>
       </c>
@@ -9181,7 +9199,7 @@
         <v>-10.60639064705564</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C7">
         <v>14000</v>
       </c>
@@ -9203,7 +9221,7 @@
         <v>-13034.940154857992</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>102</v>
       </c>
@@ -9232,7 +9250,7 @@
         <v>-5.2757114382118635</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>78</v>
       </c>
@@ -9240,12 +9258,12 @@
         <v>394716</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="18" t="s">
         <v>0</v>
       </c>
@@ -9295,7 +9313,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="15" t="s">
         <v>84</v>
       </c>
@@ -9346,7 +9364,7 @@
         <v>1.0667868110000001</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="15" t="s">
         <v>84</v>
       </c>
@@ -9397,7 +9415,7 @@
         <v>0.93243811712477798</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
         <v>84</v>
       </c>
@@ -9448,7 +9466,7 @@
         <v>0.84334790223742195</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="15" t="s">
         <v>84</v>
       </c>
@@ -9499,7 +9517,7 @@
         <v>0.77781898176327602</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17" s="15" t="s">
         <v>84</v>
       </c>
@@ -9550,7 +9568,7 @@
         <v>0.74298988026741397</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A18" s="15" t="s">
         <v>84</v>
       </c>
@@ -9601,7 +9619,7 @@
         <v>1.0717494293005001</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A19" s="15" t="s">
         <v>84</v>
       </c>
@@ -9652,7 +9670,7 @@
         <v>0.85971724445347397</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A20" s="15" t="s">
         <v>84</v>
       </c>
@@ -9703,7 +9721,7 @@
         <v>0.85637371278832397</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A21" s="15" t="s">
         <v>84</v>
       </c>
@@ -9754,7 +9772,7 @@
         <v>0.75177719391388198</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A22" s="15" t="s">
         <v>84</v>
       </c>

</xml_diff>

<commit_message>
TOU8 baseline and RTP README
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4CF949F-2DE2-4255-AD39-14C4033E85C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5598CEA7-4AA9-4BA9-BA2A-1A007AAC02AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -50,7 +50,6 @@
     <author>tc={0CE66D44-40D7-4762-8700-23B9C4E639CE}</author>
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
     <author>tc={F9308CF0-AB74-4ABB-91B6-7382ECEADD39}</author>
-    <author>tc={B08B550A-B779-4CE5-A29D-4C76A4C93C7E}</author>
     <author>tc={B12FED98-6BE9-4BE2-A887-4CF314FA442B}</author>
     <author>tc={7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}</author>
     <author>tc={B7EDEAAD-67C9-4693-A0FC-570282E02182}</author>
@@ -165,17 +164,7 @@
     Summer week = hot summer weekdays + high weekends</t>
       </text>
     </comment>
-    <comment ref="T51" authorId="12" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Don’t think I trust these metrics. Would have to re-run if we want to provide that number for this rate structure
-Reply:
-    The baseline costs have to be updated in accordance with the demand structure type</t>
-      </text>
-    </comment>
-    <comment ref="A60" authorId="13" shapeId="0" xr:uid="{B12FED98-6BE9-4BE2-A887-4CF314FA442B}">
+    <comment ref="A60" authorId="12" shapeId="0" xr:uid="{B12FED98-6BE9-4BE2-A887-4CF314FA442B}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -183,7 +172,7 @@
     Wrong baseline power was used</t>
       </text>
     </comment>
-    <comment ref="A61" authorId="14" shapeId="0" xr:uid="{7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}">
+    <comment ref="A61" authorId="13" shapeId="0" xr:uid="{7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -191,7 +180,7 @@
     Old solution where there is only one plant shutdown.</t>
       </text>
     </comment>
-    <comment ref="A62" authorId="15" shapeId="0" xr:uid="{B7EDEAAD-67C9-4693-A0FC-570282E02182}">
+    <comment ref="A62" authorId="14" shapeId="0" xr:uid="{B7EDEAAD-67C9-4693-A0FC-570282E02182}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -199,7 +188,7 @@
     Solution where there is a shutdown for all peak hours</t>
       </text>
     </comment>
-    <comment ref="A63" authorId="16" shapeId="0" xr:uid="{0EBBD83F-AB64-4248-87E6-B99F88EE5F88}">
+    <comment ref="A63" authorId="15" shapeId="0" xr:uid="{0EBBD83F-AB64-4248-87E6-B99F88EE5F88}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -207,7 +196,7 @@
     Only one plant shutdown allowed</t>
       </text>
     </comment>
-    <comment ref="A68" authorId="17" shapeId="0" xr:uid="{8E704477-0437-40A7-B175-85F6EA0FB52A}">
+    <comment ref="A68" authorId="16" shapeId="0" xr:uid="{8E704477-0437-40A7-B175-85F6EA0FB52A}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -215,7 +204,7 @@
     Including this as the final result</t>
       </text>
     </comment>
-    <comment ref="L69" authorId="18" shapeId="0" xr:uid="{9BC5A461-E691-49A7-9AA5-314B7AD6B728}">
+    <comment ref="L69" authorId="17" shapeId="0" xr:uid="{9BC5A461-E691-49A7-9AA5-314B7AD6B728}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -223,7 +212,7 @@
     Just some random lower recovery periods</t>
       </text>
     </comment>
-    <comment ref="A76" authorId="19" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
+    <comment ref="A76" authorId="18" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -232,7 +221,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="A83" authorId="20" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
+    <comment ref="A83" authorId="19" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -240,7 +229,7 @@
     Pretty sure this solution is wrong, but I don’t think I need this case for the paper</t>
       </text>
     </comment>
-    <comment ref="A89" authorId="21" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A89" authorId="20" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -248,7 +237,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="A101" authorId="22" shapeId="0" xr:uid="{3B63C6BF-9DE1-4172-A721-F97EE0406603}">
+    <comment ref="A101" authorId="21" shapeId="0" xr:uid="{3B63C6BF-9DE1-4172-A721-F97EE0406603}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -256,7 +245,7 @@
     2.5x higher brine costs (1.08$/m3)</t>
       </text>
     </comment>
-    <comment ref="A104" authorId="23" shapeId="0" xr:uid="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
+    <comment ref="A104" authorId="22" shapeId="0" xr:uid="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -264,7 +253,7 @@
     5x brine costs (2.15 $/m3)</t>
       </text>
     </comment>
-    <comment ref="A107" authorId="24" shapeId="0" xr:uid="{9D93D39A-4E12-4E91-8443-F39D5B5EA779}">
+    <comment ref="A107" authorId="23" shapeId="0" xr:uid="{9D93D39A-4E12-4E91-8443-F39D5B5EA779}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -272,7 +261,7 @@
     Working Hours = 8 AM to 5 PM</t>
       </text>
     </comment>
-    <comment ref="A112" authorId="25" shapeId="0" xr:uid="{9585276E-E9B8-4AFF-9F58-E3ADC73D024E}">
+    <comment ref="A112" authorId="24" shapeId="0" xr:uid="{9585276E-E9B8-4AFF-9F58-E3ADC73D024E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -280,7 +269,7 @@
     Five Shutdowns</t>
       </text>
     </comment>
-    <comment ref="T120" authorId="26" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T120" authorId="25" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -1819,12 +1808,6 @@
   <threadedComment ref="A51" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
     <text>Summer week = hot summer weekdays + high weekends</text>
   </threadedComment>
-  <threadedComment ref="T51" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
-    <text>Don’t think I trust these metrics. Would have to re-run if we want to provide that number for this rate structure</text>
-  </threadedComment>
-  <threadedComment ref="T51" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
-    <text>The baseline costs have to be updated in accordance with the demand structure type</text>
-  </threadedComment>
   <threadedComment ref="A60" dT="2026-07-21T19:50:00.59" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B12FED98-6BE9-4BE2-A887-4CF314FA442B}">
     <text>Wrong baseline power was used</text>
   </threadedComment>
@@ -1961,22 +1944,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
   <dimension ref="A1:V123"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.6328125" customWidth="1"/>
-    <col min="3" max="3" width="10.81640625" customWidth="1"/>
+    <col min="1" max="1" width="9.61328125" customWidth="1"/>
+    <col min="3" max="3" width="10.84375" customWidth="1"/>
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7265625" customWidth="1"/>
-    <col min="9" max="9" width="9.08984375" customWidth="1"/>
-    <col min="11" max="11" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.54296875" customWidth="1"/>
-    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.81640625" customWidth="1"/>
+    <col min="5" max="5" width="10.23046875" customWidth="1"/>
+    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.69140625" customWidth="1"/>
+    <col min="9" max="9" width="9.07421875" customWidth="1"/>
+    <col min="11" max="11" width="10.84375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.53515625" customWidth="1"/>
+    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1987,7 +1970,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2055,7 +2038,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -2119,7 +2102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -2183,14 +2166,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G5" s="4"/>
       <c r="K5" s="10">
         <f>K4+L4+M4</f>
         <v>85444.512881154791</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -2254,7 +2237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -2318,10 +2301,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -2385,7 +2368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2449,10 +2432,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -2516,7 +2499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -2580,10 +2563,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2645,7 +2628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2701,10 +2684,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2768,7 +2751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2832,7 +2815,7 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="K20">
@@ -2841,7 +2824,7 @@
       </c>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2852,7 +2835,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2916,10 +2899,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2983,7 +2966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -3053,11 +3036,11 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -3121,7 +3104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -3185,10 +3168,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -3252,7 +3235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -3322,7 +3305,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -3392,7 +3375,7 @@
         <v>277.67302057784298</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A33" s="26" t="s">
         <v>45</v>
       </c>
@@ -3475,19 +3458,19 @@
         <v>200.18128127969257</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="K34" s="10"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -3551,7 +3534,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -3615,12 +3598,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A38" s="7"/>
       <c r="B38" s="2"/>
       <c r="S38" s="2"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A39" s="3" t="s">
         <v>20</v>
       </c>
@@ -3687,7 +3670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A40" s="3" t="s">
         <v>22</v>
       </c>
@@ -3757,20 +3740,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3834,15 +3817,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A46" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -3912,13 +3895,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A49" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A50" s="2" t="s">
         <v>20</v>
       </c>
@@ -3966,7 +3949,7 @@
         <v>0</v>
       </c>
       <c r="P50">
-        <f t="shared" ref="P50:P56" si="11">D50+$P$1</f>
+        <f t="shared" ref="P50:P57" si="11">D50+$P$1</f>
         <v>238413.66244470741</v>
       </c>
       <c r="Q50">
@@ -3982,11 +3965,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A51" s="2" t="s">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A51" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C51">
@@ -3994,63 +3977,66 @@
       </c>
       <c r="D51">
         <f>J51+K51+L51+M51+N51</f>
-        <v>188012.7674304971</v>
+        <v>182278.61424564509</v>
       </c>
       <c r="E51">
-        <v>282179.67123287602</v>
+        <v>282190.859999999</v>
       </c>
       <c r="F51">
-        <v>1.09353178385</v>
+        <v>1.071688712182</v>
       </c>
       <c r="G51">
-        <v>89520.694507565597</v>
+        <v>84096.123187821693</v>
       </c>
       <c r="H51">
-        <v>6971.3813103080802</v>
+        <v>6548.9454112036401</v>
       </c>
       <c r="I51">
-        <v>5083.8680235841202</v>
+        <v>4775.8073570242204</v>
       </c>
       <c r="J51">
-        <v>101575.943841457</v>
+        <v>95420.875956049596</v>
       </c>
       <c r="K51">
-        <v>50843.184005923598</v>
+        <v>50845.200000000099</v>
       </c>
       <c r="L51">
-        <v>15303.798385783</v>
+        <v>15304.405199999899</v>
       </c>
       <c r="M51">
-        <v>19297.5304894482</v>
+        <v>19298.29566</v>
       </c>
       <c r="N51">
-        <v>992.31070788530405</v>
+        <v>1409.83742959549</v>
       </c>
       <c r="O51">
         <v>0</v>
       </c>
       <c r="P51">
         <f t="shared" si="11"/>
-        <v>308572.43924949365</v>
+        <v>302838.28606464161</v>
       </c>
       <c r="Q51">
-        <v>1106.4527933521999</v>
+        <v>1101.77087397171</v>
       </c>
       <c r="R51">
-        <v>3451.9307168288801</v>
+        <v>38.493172752110603</v>
       </c>
       <c r="S51">
-        <v>20.547206647791</v>
+        <v>0.22912602828637299</v>
       </c>
       <c r="T51">
-        <v>-14.696886263168601</v>
-      </c>
-    </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
+        <v>123.174719446704</v>
+      </c>
+      <c r="U51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A53" s="2" t="s">
         <v>20</v>
       </c>
@@ -4114,7 +4100,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A54" s="2" t="s">
         <v>22</v>
       </c>
@@ -4178,10 +4164,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A56" s="2" t="s">
         <v>20</v>
       </c>
@@ -4245,7 +4231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A57" s="5" t="s">
         <v>22</v>
       </c>
@@ -4256,7 +4242,8 @@
         <v>4</v>
       </c>
       <c r="D57">
-        <v>120512.352495367</v>
+        <f>J57+K57+L57+M57+N57</f>
+        <v>121985.71201190345</v>
       </c>
       <c r="E57">
         <v>282179.671232878</v>
@@ -4292,7 +4279,8 @@
         <v>0</v>
       </c>
       <c r="P57">
-        <v>242064.335022249</v>
+        <f t="shared" si="11"/>
+        <v>242545.38383089995</v>
       </c>
       <c r="Q57">
         <v>1460.1650793650699</v>
@@ -4313,13 +4301,13 @@
         <v>357.90412909372202</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A60" s="2" t="s">
         <v>22</v>
       </c>
@@ -4383,7 +4371,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A61" s="3" t="s">
         <v>22</v>
       </c>
@@ -4448,7 +4436,7 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A62" s="5" t="s">
         <v>22</v>
       </c>
@@ -4518,7 +4506,7 @@
         <v>278.17977348178903</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -4588,7 +4576,7 @@
         <v>107.018147807505</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A64" s="26" t="s">
         <v>44</v>
       </c>
@@ -4671,19 +4659,19 @@
         <v>-171.16162567428404</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A66" s="9"/>
       <c r="B66" s="9"/>
       <c r="C66" s="9"/>
       <c r="D66" s="13"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A67" s="26" t="s">
         <v>60</v>
       </c>
@@ -4691,7 +4679,7 @@
       <c r="C67" s="26"/>
       <c r="D67" s="10"/>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A68" s="5" t="s">
         <v>22</v>
       </c>
@@ -4761,7 +4749,7 @@
         <v>350.36946039055402</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A69" s="26" t="s">
         <v>61</v>
       </c>
@@ -4820,7 +4808,7 @@
         <v>133.12347700700047</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A70" s="9"/>
       <c r="B70" s="9"/>
       <c r="C70" s="9"/>
@@ -4841,13 +4829,13 @@
       <c r="O70" s="10"/>
       <c r="P70" s="10"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A71" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G71" s="4"/>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -4859,7 +4847,7 @@
       </c>
       <c r="G72" s="4"/>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
         <v>22</v>
       </c>
@@ -4923,13 +4911,13 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
       <c r="G74" s="4"/>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A75" s="3" t="s">
         <v>20</v>
       </c>
@@ -4941,7 +4929,7 @@
       </c>
       <c r="G75" s="4"/>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
         <v>22</v>
       </c>
@@ -5010,7 +4998,7 @@
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="D77">
@@ -5090,12 +5078,12 @@
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A78" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A79" s="3" t="s">
         <v>20</v>
       </c>
@@ -5159,7 +5147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A80" s="3" t="s">
         <v>22</v>
       </c>
@@ -5223,10 +5211,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A81" s="1"/>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
         <v>20</v>
       </c>
@@ -5284,7 +5272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A83" s="2" t="s">
         <v>22</v>
       </c>
@@ -5348,7 +5336,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
         <v>20</v>
       </c>
@@ -5406,7 +5394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
         <v>22</v>
       </c>
@@ -5476,7 +5464,7 @@
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.4">
       <c r="D87">
         <f>D86-D80</f>
         <v>-4018.7603482047853</v>
@@ -5526,13 +5514,13 @@
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A88" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G88" s="4"/>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
         <v>22</v>
       </c>
@@ -5596,7 +5584,7 @@
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
         <v>22</v>
       </c>
@@ -5640,8 +5628,8 @@
         <v>36</v>
       </c>
     </row>
-    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.4"/>
+    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A92" s="1" t="s">
         <v>26</v>
       </c>
@@ -5662,7 +5650,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
         <v>0</v>
       </c>
@@ -5724,10 +5712,10 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G94" s="4"/>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A95" t="s">
         <v>20</v>
       </c>
@@ -5797,7 +5785,7 @@
         <v>319.37310450388202</v>
       </c>
     </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A96" s="3" t="s">
         <v>20</v>
       </c>
@@ -5842,16 +5830,16 @@
         <v>36</v>
       </c>
     </row>
-    <row r="97" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A97" s="2"/>
       <c r="G97" s="4"/>
     </row>
-    <row r="99" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A99" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A100" t="s">
         <v>22</v>
       </c>
@@ -5904,7 +5892,7 @@
         <v>265201.24508552696</v>
       </c>
     </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A101" t="s">
         <v>22</v>
       </c>
@@ -5974,13 +5962,13 @@
         <v>290.07670650869801</v>
       </c>
     </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:22" x14ac:dyDescent="0.4">
       <c r="K102">
         <f>SUM(K100:M100)-SUM(K101:M101)</f>
         <v>-750.09243586547382</v>
       </c>
     </row>
-    <row r="103" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A103" t="s">
         <v>22</v>
       </c>
@@ -6030,7 +6018,7 @@
         <v>303282.7899059637</v>
       </c>
     </row>
-    <row r="104" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A104" t="s">
         <v>22</v>
       </c>
@@ -6100,19 +6088,19 @@
         <v>351.71871156820202</v>
       </c>
     </row>
-    <row r="105" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:22" x14ac:dyDescent="0.4">
       <c r="K105" s="13">
         <f>SUM(K103:M103)-SUM(K104:M104)</f>
         <v>-831.26776848098962</v>
       </c>
     </row>
-    <row r="106" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A106" s="1" t="s">
         <v>65</v>
       </c>
       <c r="K106" s="13"/>
     </row>
-    <row r="107" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A107" t="s">
         <v>22</v>
       </c>
@@ -6182,7 +6170,7 @@
         <v>359.195907759661</v>
       </c>
     </row>
-    <row r="108" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A108" t="s">
         <v>22</v>
       </c>
@@ -6252,7 +6240,7 @@
         <v>331.01860370537798</v>
       </c>
     </row>
-    <row r="109" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:22" x14ac:dyDescent="0.4">
       <c r="D109" s="13">
         <f>D108-D31</f>
         <v>870.81314264753019</v>
@@ -6298,7 +6286,7 @@
         <v>-2.9942133752499558</v>
       </c>
     </row>
-    <row r="110" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:22" x14ac:dyDescent="0.4">
       <c r="D110" s="13"/>
       <c r="E110" s="13"/>
       <c r="F110" s="13"/>
@@ -6311,7 +6299,7 @@
       <c r="M110" s="13"/>
       <c r="N110" s="13"/>
     </row>
-    <row r="111" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A111" s="1" t="s">
         <v>66</v>
       </c>
@@ -6327,7 +6315,7 @@
       <c r="M111" s="13"/>
       <c r="N111" s="13"/>
     </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A112" t="s">
         <v>22</v>
       </c>
@@ -6397,7 +6385,7 @@
         <v>300.72865279776499</v>
       </c>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.4">
       <c r="D113" s="12">
         <f>(D112-D4)</f>
         <v>-7531.9083775022591</v>
@@ -6413,7 +6401,7 @@
       <c r="M113" s="13"/>
       <c r="N113" s="13"/>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.4">
       <c r="D114" s="13"/>
       <c r="E114" s="13"/>
       <c r="F114" s="13"/>
@@ -6426,12 +6414,12 @@
       <c r="M114" s="13"/>
       <c r="N114" s="13"/>
     </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A115" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A116" t="s">
         <v>32</v>
       </c>
@@ -6442,7 +6430,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A117">
         <v>20</v>
       </c>
@@ -6506,7 +6494,7 @@
         <v>0.12591688076390301</v>
       </c>
     </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A118">
         <v>20</v>
       </c>
@@ -6570,7 +6558,7 @@
         <v>0.14758705239613301</v>
       </c>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A119">
         <v>20</v>
       </c>
@@ -6634,7 +6622,7 @@
         <v>-0.25983751983286502</v>
       </c>
     </row>
-    <row r="120" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A120">
         <v>20</v>
       </c>
@@ -6698,7 +6686,7 @@
         <v>0.28049716262959101</v>
       </c>
     </row>
-    <row r="121" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A121" s="3">
         <v>20</v>
       </c>
@@ -6762,7 +6750,7 @@
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A122">
         <v>20</v>
       </c>
@@ -6826,7 +6814,7 @@
         <v>0.46004655114715598</v>
       </c>
     </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A123">
         <v>20</v>
       </c>
@@ -6906,20 +6894,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA993591-8C1F-4C7B-A75D-E9726DFB461B}">
   <dimension ref="A2:P31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="12.81640625" customWidth="1"/>
-    <col min="3" max="3" width="11.36328125" customWidth="1"/>
-    <col min="4" max="4" width="15.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.84375" customWidth="1"/>
+    <col min="3" max="3" width="11.3828125" customWidth="1"/>
+    <col min="4" max="4" width="15.53515625" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="17.08984375" customWidth="1"/>
-    <col min="7" max="7" width="15.26953125" customWidth="1"/>
-    <col min="8" max="8" width="13.26953125" customWidth="1"/>
-    <col min="9" max="11" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.07421875" customWidth="1"/>
+    <col min="7" max="7" width="15.23046875" customWidth="1"/>
+    <col min="8" max="8" width="13.23046875" customWidth="1"/>
+    <col min="9" max="11" width="11.3828125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -6958,12 +6946,12 @@
       </c>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -7002,7 +6990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="D5" s="10"/>
@@ -7014,7 +7002,7 @@
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>48</v>
       </c>
@@ -7031,7 +7019,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -7071,7 +7059,7 @@
       </c>
       <c r="M7" s="11"/>
     </row>
-    <row r="8" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D8" s="10">
         <f t="shared" ref="D8:K8" si="0">D7-D4</f>
         <v>759.28494035729091</v>
@@ -7106,7 +7094,7 @@
       </c>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>62</v>
       </c>
@@ -7120,7 +7108,7 @@
       <c r="K9" s="10"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B10" t="s">
         <v>21</v>
       </c>
@@ -7156,7 +7144,7 @@
       </c>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
       <c r="D11">
         <f>(34653-H10-I11+wrd_pricetater_flex_type_summar!K5+L10)/34653</f>
         <v>0.17154119896168271</v>
@@ -7173,7 +7161,7 @@
       <c r="K11" s="10"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>49</v>
       </c>
@@ -7187,7 +7175,7 @@
       <c r="K12" s="10"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A13" s="3" t="s">
         <v>22</v>
       </c>
@@ -7227,7 +7215,7 @@
       </c>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="D14" s="10"/>
@@ -7240,7 +7228,7 @@
       <c r="K14" s="10"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>46</v>
       </c>
@@ -7253,7 +7241,7 @@
       <c r="J15" s="10"/>
       <c r="K15" s="10"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -7292,7 +7280,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
       <c r="D17">
         <f>(34653-H16-I17+wrd_pricetater_flex_type_summar!K5+L16)/34653</f>
         <v>0.38932217950875497</v>
@@ -7302,7 +7290,7 @@
         <v>87792.098602195503</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
         <v>57</v>
       </c>
@@ -7341,7 +7329,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -7349,7 +7337,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>52</v>
       </c>
@@ -7387,7 +7375,7 @@
       </c>
       <c r="L23" s="10"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>55</v>
       </c>
@@ -7425,7 +7413,7 @@
       </c>
       <c r="L25" s="10"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -7462,7 +7450,7 @@
         <v>-476.58002357000078</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -7499,7 +7487,7 @@
         <v>174.37684745549996</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>58</v>
       </c>
@@ -7545,25 +7533,25 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BC34AED-31C3-47D6-9398-9693457BF528}">
   <dimension ref="A1:AB19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="26.90625" customWidth="1"/>
-    <col min="2" max="2" width="14.7265625" customWidth="1"/>
-    <col min="3" max="3" width="12.08984375" customWidth="1"/>
+    <col min="1" max="1" width="26.921875" customWidth="1"/>
+    <col min="2" max="2" width="14.69140625" customWidth="1"/>
+    <col min="3" max="3" width="12.07421875" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="8.54296875" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="15.08984375" customWidth="1"/>
-    <col min="8" max="8" width="10.1796875" customWidth="1"/>
-    <col min="9" max="9" width="11.36328125" customWidth="1"/>
+    <col min="5" max="5" width="8.53515625" customWidth="1"/>
+    <col min="6" max="6" width="11.3828125" customWidth="1"/>
+    <col min="7" max="7" width="15.07421875" customWidth="1"/>
+    <col min="8" max="8" width="10.15234375" customWidth="1"/>
+    <col min="9" max="9" width="11.3828125" customWidth="1"/>
     <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.90625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="10.7265625" customWidth="1"/>
-    <col min="28" max="28" width="13.81640625" customWidth="1"/>
+    <col min="11" max="11" width="16.921875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.69140625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.69140625" customWidth="1"/>
+    <col min="28" max="28" width="13.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.4">
       <c r="G1">
         <v>121507.92454383519</v>
       </c>
@@ -7571,7 +7559,7 @@
         <v>34653.411662680403</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>67</v>
       </c>
@@ -7657,7 +7645,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>0</v>
       </c>
@@ -7747,7 +7735,7 @@
         <v>0.21734969274652002</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>0.215</v>
       </c>
@@ -7837,7 +7825,7 @@
         <v>0.14991564378830438</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>0.43</v>
       </c>
@@ -7928,7 +7916,7 @@
         <v>0.1072768553096176</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>0.86</v>
       </c>
@@ -8019,7 +8007,7 @@
         <v>0.1072768553096176</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>1.29</v>
       </c>
@@ -8110,14 +8098,14 @@
         <v>0.1072768553096176</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="21" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:28" s="21" customFormat="1" x14ac:dyDescent="0.4">
       <c r="D8" s="22"/>
       <c r="E8" s="22"/>
       <c r="Q8" s="23"/>
       <c r="AA8" s="24"/>
       <c r="AB8" s="25"/>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>0</v>
       </c>
@@ -8224,7 +8212,7 @@
         <v>0.53535589967557295</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>0.215</v>
       </c>
@@ -8331,7 +8319,7 @@
         <v>0.46792185071735731</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>0.43</v>
       </c>
@@ -8422,7 +8410,7 @@
         <v>0.40263355404451467</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>0.86</v>
       </c>
@@ -8512,7 +8500,7 @@
         <v>0.36082050708979968</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>1.29</v>
       </c>
@@ -8603,11 +8591,11 @@
         <v>0.33396366478241479</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="21" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:28" s="21" customFormat="1" x14ac:dyDescent="0.4">
       <c r="AA14" s="24"/>
       <c r="AB14" s="25"/>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A15" s="2">
         <v>0</v>
       </c>
@@ -8694,10 +8682,10 @@
       </c>
       <c r="AB15" s="12">
         <f>(wrd_pricetater_flex_type_summar!$D$51-G15)/wrd_pricetater_flex_type_summar!$J$51</f>
-        <v>0.67280721058037529</v>
-      </c>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
+        <v>0.65611296926286822</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A16" s="2">
         <v>0.215</v>
       </c>
@@ -8784,10 +8772,10 @@
       </c>
       <c r="AB16" s="12">
         <f>(wrd_pricetater_flex_type_summar!$D$51-G16)/wrd_pricetater_flex_type_summar!$J$51</f>
-        <v>0.64784363750995022</v>
-      </c>
-    </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.35">
+        <v>0.62953913548825957</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A17" s="2">
         <v>0.43</v>
       </c>
@@ -8875,10 +8863,10 @@
       </c>
       <c r="AB17" s="12">
         <f>(wrd_pricetater_flex_type_summar!$D$51-G17)/wrd_pricetater_flex_type_summar!$J$51</f>
-        <v>0.63256386175391488</v>
-      </c>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.35">
+        <v>0.61327374671924462</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A18" s="2">
         <v>0.86</v>
       </c>
@@ -8965,10 +8953,10 @@
       </c>
       <c r="AB18" s="12">
         <f>(wrd_pricetater_flex_type_summar!$D$51-G18)/wrd_pricetater_flex_type_summar!$J$51</f>
-        <v>0.58579049127122573</v>
-      </c>
-    </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.35">
+        <v>0.56348328728546615</v>
+      </c>
+    </row>
+    <row r="19" spans="1:28" x14ac:dyDescent="0.4">
       <c r="A19" s="2">
         <v>1.29</v>
       </c>
@@ -9055,7 +9043,7 @@
       </c>
       <c r="AB19" s="12">
         <f>(wrd_pricetater_flex_type_summar!$D$51-G19)/wrd_pricetater_flex_type_summar!$J$51</f>
-        <v>0.54058832177700888</v>
+        <v>0.51536537824246598</v>
       </c>
     </row>
   </sheetData>
@@ -9068,24 +9056,24 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FD55A87-71DC-49C4-874A-7F05794F4461}">
   <dimension ref="A3:P22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="12.6328125" customWidth="1"/>
-    <col min="3" max="3" width="9.7265625" customWidth="1"/>
-    <col min="4" max="4" width="12.453125" customWidth="1"/>
+    <col min="2" max="2" width="12.61328125" customWidth="1"/>
+    <col min="3" max="3" width="9.69140625" customWidth="1"/>
+    <col min="4" max="4" width="12.4609375" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="20.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.26953125" customWidth="1"/>
-    <col min="8" max="8" width="18.54296875" customWidth="1"/>
-    <col min="9" max="9" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.08984375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.26953125" customWidth="1"/>
-    <col min="13" max="13" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.1796875" customWidth="1"/>
+    <col min="6" max="6" width="20.921875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.23046875" customWidth="1"/>
+    <col min="8" max="8" width="18.53515625" customWidth="1"/>
+    <col min="9" max="9" width="20.15234375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.07421875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.3828125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.23046875" customWidth="1"/>
+    <col min="13" max="13" width="9.3828125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.15234375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
       <c r="C3" t="s">
         <v>76</v>
       </c>
@@ -9108,7 +9096,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
       <c r="B4" t="s">
         <v>101</v>
       </c>
@@ -9137,7 +9125,7 @@
         <v>-4.0410044714229976</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
       <c r="C5">
         <v>10000</v>
       </c>
@@ -9159,7 +9147,7 @@
         <v>-12815.109372157822</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.4">
       <c r="C6">
         <v>12000</v>
       </c>
@@ -9185,7 +9173,7 @@
         <v>-10.60639064705564</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.4">
       <c r="C7">
         <v>14000</v>
       </c>
@@ -9207,7 +9195,7 @@
         <v>-13034.940154857992</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.4">
       <c r="B8" t="s">
         <v>102</v>
       </c>
@@ -9236,7 +9224,7 @@
         <v>-5.2757114382118635</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.4">
       <c r="B9" t="s">
         <v>78</v>
       </c>
@@ -9244,12 +9232,12 @@
         <v>394716</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A12" s="18" t="s">
         <v>0</v>
       </c>
@@ -9299,7 +9287,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A13" s="15" t="s">
         <v>84</v>
       </c>
@@ -9350,7 +9338,7 @@
         <v>1.0667868110000001</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A14" s="15" t="s">
         <v>84</v>
       </c>
@@ -9401,7 +9389,7 @@
         <v>0.93243811712477798</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A15" s="15" t="s">
         <v>84</v>
       </c>
@@ -9452,7 +9440,7 @@
         <v>0.84334790223742195</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A16" s="15" t="s">
         <v>84</v>
       </c>
@@ -9503,7 +9491,7 @@
         <v>0.77781898176327602</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A17" s="15" t="s">
         <v>84</v>
       </c>
@@ -9554,7 +9542,7 @@
         <v>0.74298988026741397</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A18" s="15" t="s">
         <v>84</v>
       </c>
@@ -9605,7 +9593,7 @@
         <v>1.0717494293005001</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A19" s="15" t="s">
         <v>84</v>
       </c>
@@ -9656,7 +9644,7 @@
         <v>0.85971724445347397</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A20" s="15" t="s">
         <v>84</v>
       </c>
@@ -9707,7 +9695,7 @@
         <v>0.85637371278832397</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A21" s="15" t="s">
         <v>84</v>
       </c>
@@ -9758,7 +9746,7 @@
         <v>0.75177719391388198</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A22" s="15" t="s">
         <v>84</v>
       </c>

</xml_diff>

<commit_message>
Updating TOU8 files and creating new figures for the paper
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5598CEA7-4AA9-4BA9-BA2A-1A007AAC02AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A09BA11-C389-447D-B5FD-2BEDC67CF040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -57,6 +57,7 @@
     <author>tc={8E704477-0437-40A7-B175-85F6EA0FB52A}</author>
     <author>tc={9BC5A461-E691-49A7-9AA5-314B7AD6B728}</author>
     <author>tc={FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}</author>
+    <author>tc={72AFD5EA-5AA9-4CD2-944C-D32BC94D67D2}</author>
     <author>tc={4644E393-F522-4E79-88BA-041770B595A7}</author>
     <author>tc={9FF6B967-6104-43AC-8EED-15C48C9ACCA9}</author>
     <author>tc={3B63C6BF-9DE1-4172-A721-F97EE0406603}</author>
@@ -221,7 +222,15 @@
 </t>
       </text>
     </comment>
-    <comment ref="A83" authorId="19" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
+    <comment ref="A78" authorId="19" shapeId="0" xr:uid="{72AFD5EA-5AA9-4CD2-944C-D32BC94D67D2}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    If RED, result is using the 2026 rate, but I’m updating to the 2023 version</t>
+      </text>
+    </comment>
+    <comment ref="A83" authorId="20" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -229,7 +238,7 @@
     Pretty sure this solution is wrong, but I don’t think I need this case for the paper</t>
       </text>
     </comment>
-    <comment ref="A89" authorId="20" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A89" authorId="21" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -237,7 +246,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="A101" authorId="21" shapeId="0" xr:uid="{3B63C6BF-9DE1-4172-A721-F97EE0406603}">
+    <comment ref="A101" authorId="22" shapeId="0" xr:uid="{3B63C6BF-9DE1-4172-A721-F97EE0406603}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -245,7 +254,7 @@
     2.5x higher brine costs (1.08$/m3)</t>
       </text>
     </comment>
-    <comment ref="A104" authorId="22" shapeId="0" xr:uid="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
+    <comment ref="A104" authorId="23" shapeId="0" xr:uid="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -253,7 +262,7 @@
     5x brine costs (2.15 $/m3)</t>
       </text>
     </comment>
-    <comment ref="A107" authorId="23" shapeId="0" xr:uid="{9D93D39A-4E12-4E91-8443-F39D5B5EA779}">
+    <comment ref="A107" authorId="24" shapeId="0" xr:uid="{9D93D39A-4E12-4E91-8443-F39D5B5EA779}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -261,7 +270,7 @@
     Working Hours = 8 AM to 5 PM</t>
       </text>
     </comment>
-    <comment ref="A112" authorId="24" shapeId="0" xr:uid="{9585276E-E9B8-4AFF-9F58-E3ADC73D024E}">
+    <comment ref="A112" authorId="25" shapeId="0" xr:uid="{9585276E-E9B8-4AFF-9F58-E3ADC73D024E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -269,7 +278,7 @@
     Five Shutdowns</t>
       </text>
     </comment>
-    <comment ref="T120" authorId="25" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T120" authorId="26" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -808,7 +817,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -975,6 +984,20 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="35">
@@ -1354,7 +1377,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1388,6 +1411,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1830,6 +1854,9 @@
     <text xml:space="preserve">This should be the same as the other DR solution, except for the demand response revenue
 </text>
   </threadedComment>
+  <threadedComment ref="A78" dT="2026-09-11T22:19:30.96" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{72AFD5EA-5AA9-4CD2-944C-D32BC94D67D2}">
+    <text>If RED, result is using the 2026 rate, but I’m updating to the 2023 version</text>
+  </threadedComment>
   <threadedComment ref="A83" dT="2026-07-21T19:23:55.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4644E393-F522-4E79-88BA-041770B595A7}">
     <text>Pretty sure this solution is wrong, but I don’t think I need this case for the paper</text>
   </threadedComment>
@@ -4301,6 +4328,12 @@
         <v>357.90412909372202</v>
       </c>
     </row>
+    <row r="58" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="K58">
+        <f>K57+L57+M57-(K51+L51+M51)</f>
+        <v>5389.7553551421151</v>
+      </c>
+    </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A59" s="1" t="s">
         <v>30</v>
@@ -5084,10 +5117,10 @@
       </c>
     </row>
     <row r="79" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A79" s="3" t="s">
+      <c r="A79" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B79" s="3" t="s">
+      <c r="B79" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C79">
@@ -5148,10 +5181,10 @@
       </c>
     </row>
     <row r="80" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A80" s="3" t="s">
+      <c r="A80" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B80" s="3" t="s">
+      <c r="B80" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C80">
@@ -5159,47 +5192,47 @@
       </c>
       <c r="D80">
         <f>J80+K80+L80+M80+N80</f>
-        <v>125763.55741733511</v>
+        <v>124337.62912011228</v>
       </c>
       <c r="E80">
-        <v>282179.67125180899</v>
+        <v>282190.859999999</v>
       </c>
       <c r="F80">
-        <v>0.87293045648394496</v>
+        <v>0.86636319198077105</v>
       </c>
       <c r="G80">
-        <v>22626.697961956499</v>
+        <v>22795.571059233</v>
       </c>
       <c r="H80">
-        <v>7102.5767129513297</v>
+        <v>5233.0127982051599</v>
       </c>
       <c r="I80">
-        <v>9597.4591384874802</v>
+        <v>9451.3069638763409</v>
       </c>
       <c r="J80">
-        <v>39326.733813395302</v>
+        <v>37479.890821314497</v>
       </c>
       <c r="K80">
-        <v>50843.184011688398</v>
+        <v>50845.200002362697</v>
       </c>
       <c r="L80">
-        <v>15303.798393134501</v>
+        <v>15304.4052063494</v>
       </c>
       <c r="M80">
-        <v>19297.530491231599</v>
+        <v>19298.295660490199</v>
       </c>
       <c r="N80">
-        <v>992.31070788530405</v>
+        <v>1409.83742959549</v>
       </c>
       <c r="O80">
         <v>0</v>
       </c>
       <c r="P80">
         <f t="shared" si="17"/>
-        <v>246323.22923633162</v>
+        <v>244897.3009391088</v>
       </c>
       <c r="Q80">
-        <v>1127.27501714903</v>
+        <v>1127.3472943468801</v>
       </c>
       <c r="R80">
         <v>0</v>
@@ -5212,13 +5245,14 @@
       </c>
     </row>
     <row r="81" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A81" s="1"/>
+      <c r="A81" s="27"/>
+      <c r="B81" s="2"/>
     </row>
     <row r="82" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A82" t="s">
+      <c r="A82" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B82" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C82">
@@ -5336,11 +5370,15 @@
         <v>1.0959871186973</v>
       </c>
     </row>
+    <row r="84" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A84" s="2"/>
+      <c r="B84" s="2"/>
+    </row>
     <row r="85" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A85" t="s">
+      <c r="A85" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B85" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C85">
@@ -5395,10 +5433,10 @@
       </c>
     </row>
     <row r="86" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A86" t="s">
+      <c r="A86" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B86" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C86">
@@ -5406,34 +5444,34 @@
       </c>
       <c r="D86">
         <f>J86+K86+L86+M86+N86</f>
-        <v>121744.79706913032</v>
+        <v>119679.31713838593</v>
       </c>
       <c r="E86">
-        <v>282179.88376308198</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F86">
-        <v>0.85713546401894802</v>
+        <v>0.84981637630953</v>
       </c>
       <c r="G86">
-        <v>21291.5607898614</v>
+        <v>21259.596722088401</v>
       </c>
       <c r="H86">
-        <v>7432.3603175362596</v>
+        <v>5421.7142614628301</v>
       </c>
       <c r="I86">
-        <v>5035.2758648834497</v>
+        <v>4952.1226155222203</v>
       </c>
       <c r="J86">
-        <v>33759.196972281097</v>
+        <v>31633.433599073502</v>
       </c>
       <c r="K86">
-        <v>51128.3645002267</v>
+        <v>51143.819864261903</v>
       </c>
       <c r="L86">
-        <v>16070.129576240101</v>
+        <v>16111.757255067099</v>
       </c>
       <c r="M86">
-        <v>19356.7120304526</v>
+        <v>19359.912430053599</v>
       </c>
       <c r="N86">
         <v>1430.39398992981</v>
@@ -5443,75 +5481,35 @@
       </c>
       <c r="P86">
         <f t="shared" si="19"/>
-        <v>242304.46888812684</v>
+        <v>240238.98895738245</v>
       </c>
       <c r="Q86">
-        <v>1179.61640190856</v>
+        <v>1167.9992270377099</v>
       </c>
       <c r="R86">
-        <v>13411.4010346792</v>
+        <v>12796.980451596301</v>
       </c>
       <c r="S86">
-        <v>478.97860838140201</v>
+        <v>511.87921806385202</v>
       </c>
       <c r="T86">
-        <v>0.22564405635506199</v>
+        <v>3.2717316651185699E-2</v>
       </c>
       <c r="U86">
-        <v>10550.3210016294</v>
+        <v>9062.6004208208706</v>
       </c>
       <c r="V86">
-        <v>75.359435725924598</v>
+        <v>63.374828117628397</v>
       </c>
     </row>
     <row r="87" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="D87">
-        <f>D86-D80</f>
-        <v>-4018.7603482047853</v>
-      </c>
-      <c r="E87">
-        <f t="shared" ref="E87:N87" si="20">E86-E80</f>
-        <v>0.21251127298455685</v>
-      </c>
-      <c r="F87">
-        <f t="shared" si="20"/>
-        <v>-1.5794992464996938E-2</v>
-      </c>
-      <c r="G87">
-        <f t="shared" si="20"/>
-        <v>-1335.1371720950992</v>
-      </c>
-      <c r="H87">
-        <f t="shared" si="20"/>
-        <v>329.78360458492989</v>
-      </c>
-      <c r="I87">
-        <f t="shared" si="20"/>
-        <v>-4562.1832736040305</v>
-      </c>
-      <c r="J87">
-        <f t="shared" si="20"/>
-        <v>-5567.5368411142044</v>
-      </c>
       <c r="K87">
-        <f t="shared" si="20"/>
-        <v>285.1804885383026</v>
-      </c>
-      <c r="L87">
-        <f t="shared" si="20"/>
-        <v>766.33118310559985</v>
-      </c>
-      <c r="M87">
-        <f t="shared" si="20"/>
-        <v>59.181539221001003</v>
-      </c>
-      <c r="N87">
-        <f t="shared" si="20"/>
-        <v>438.08328204450595</v>
+        <f>K86+L86+M86-(K80+L80+M80)</f>
+        <v>1167.588680180299</v>
       </c>
       <c r="P87">
         <f t="shared" si="19"/>
-        <v>116540.91147079173</v>
+        <v>120559.67181899652</v>
       </c>
     </row>
     <row r="88" spans="1:22" x14ac:dyDescent="0.4">
@@ -5763,7 +5761,7 @@
         <v>0</v>
       </c>
       <c r="P95">
-        <f t="shared" ref="P95" si="21">D95+$P$1</f>
+        <f t="shared" ref="P95" si="20">D95+$P$1</f>
         <v>242122.79075786425</v>
       </c>
       <c r="Q95">
@@ -5888,7 +5886,7 @@
         <v>0</v>
       </c>
       <c r="P100">
-        <f t="shared" ref="P100" si="22">D100+$P$1</f>
+        <f t="shared" ref="P100" si="21">D100+$P$1</f>
         <v>265201.24508552696</v>
       </c>
     </row>
@@ -5940,7 +5938,7 @@
         <v>0</v>
       </c>
       <c r="P101">
-        <f t="shared" ref="P101" si="23">D101+$P$1</f>
+        <f t="shared" ref="P101" si="22">D101+$P$1</f>
         <v>262246.28626913059</v>
       </c>
       <c r="Q101">
@@ -6014,7 +6012,7 @@
         <v>1410</v>
       </c>
       <c r="P103">
-        <f t="shared" ref="P103:P104" si="24">D103+$P$1</f>
+        <f t="shared" ref="P103:P104" si="23">D103+$P$1</f>
         <v>303282.7899059637</v>
       </c>
     </row>
@@ -6066,7 +6064,7 @@
         <v>0</v>
       </c>
       <c r="P104">
-        <f t="shared" si="24"/>
+        <f t="shared" si="23"/>
         <v>300724.39835160982</v>
       </c>
       <c r="Q104" s="4">
@@ -6148,7 +6146,7 @@
         <v>0</v>
       </c>
       <c r="P107">
-        <f t="shared" ref="P107:P108" si="25">D107+$P$1</f>
+        <f t="shared" ref="P107:P108" si="24">D107+$P$1</f>
         <v>240286.0714719703</v>
       </c>
       <c r="Q107">
@@ -6218,7 +6216,7 @@
         <v>0</v>
       </c>
       <c r="P108">
-        <f t="shared" si="25"/>
+        <f t="shared" si="24"/>
         <v>239220.90047655726</v>
       </c>
       <c r="Q108">
@@ -6246,43 +6244,43 @@
         <v>870.81314264753019</v>
       </c>
       <c r="E109" s="13">
-        <f t="shared" ref="E109:N109" si="26">E108-E31</f>
+        <f t="shared" ref="E109:N109" si="25">E108-E31</f>
         <v>15.79363181698136</v>
       </c>
       <c r="F109" s="13">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>3.0492754563130609E-3</v>
       </c>
       <c r="G109" s="13">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>270.37094434599931</v>
       </c>
       <c r="H109" s="13">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>1259.5735968278204</v>
       </c>
       <c r="I109" s="13">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>12.753618583180469</v>
       </c>
       <c r="J109" s="13">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>1542.6981597569975</v>
       </c>
       <c r="K109" s="13">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>-170.1127457354014</v>
       </c>
       <c r="L109" s="13">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>-463.96926584500034</v>
       </c>
       <c r="M109" s="13">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>-34.808792153802642</v>
       </c>
       <c r="N109" s="13">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>-2.9942133752499558</v>
       </c>
     </row>
@@ -6363,7 +6361,7 @@
         <v>0</v>
       </c>
       <c r="P112">
-        <f t="shared" ref="P112" si="27">D112+$P$1</f>
+        <f t="shared" ref="P112" si="26">D112+$P$1</f>
         <v>234535.68798532945</v>
       </c>
       <c r="Q112">
@@ -6441,7 +6439,7 @@
         <v>2</v>
       </c>
       <c r="D117">
-        <f t="shared" ref="D117:D123" si="28">J117+K117+L117+M117+N117</f>
+        <f t="shared" ref="D117:D123" si="27">J117+K117+L117+M117+N117</f>
         <v>120712.69088313227</v>
       </c>
       <c r="E117">
@@ -6478,7 +6476,7 @@
         <v>0</v>
       </c>
       <c r="P117">
-        <f t="shared" ref="P117:P123" si="29">D117+$P$1</f>
+        <f t="shared" ref="P117:P123" si="28">D117+$P$1</f>
         <v>241272.36270212877</v>
       </c>
       <c r="Q117">
@@ -6505,7 +6503,7 @@
         <v>2</v>
       </c>
       <c r="D118">
-        <f t="shared" si="28"/>
+        <f t="shared" si="27"/>
         <v>119392.42354269064</v>
       </c>
       <c r="E118">
@@ -6542,7 +6540,7 @@
         <v>0</v>
       </c>
       <c r="P118">
-        <f t="shared" si="29"/>
+        <f t="shared" si="28"/>
         <v>239952.09536168716</v>
       </c>
       <c r="Q118">
@@ -6569,7 +6567,7 @@
         <v>2</v>
       </c>
       <c r="D119">
-        <f t="shared" si="28"/>
+        <f t="shared" si="27"/>
         <v>117777.02945340994</v>
       </c>
       <c r="E119">
@@ -6606,7 +6604,7 @@
         <v>0</v>
       </c>
       <c r="P119">
-        <f t="shared" si="29"/>
+        <f t="shared" si="28"/>
         <v>238336.70127240644</v>
       </c>
       <c r="Q119">
@@ -6633,7 +6631,7 @@
         <v>2</v>
       </c>
       <c r="D120">
-        <f t="shared" si="28"/>
+        <f t="shared" si="27"/>
         <v>116625.1695160947</v>
       </c>
       <c r="E120">
@@ -6670,7 +6668,7 @@
         <v>0</v>
       </c>
       <c r="P120">
-        <f t="shared" si="29"/>
+        <f t="shared" si="28"/>
         <v>237184.84133509122</v>
       </c>
       <c r="Q120">
@@ -6697,7 +6695,7 @@
         <v>2</v>
       </c>
       <c r="D121">
-        <f t="shared" si="28"/>
+        <f t="shared" si="27"/>
         <v>115198.459983006</v>
       </c>
       <c r="E121">
@@ -6734,7 +6732,7 @@
         <v>0</v>
       </c>
       <c r="P121">
-        <f t="shared" si="29"/>
+        <f t="shared" si="28"/>
         <v>235758.13180200252</v>
       </c>
       <c r="Q121">
@@ -6761,7 +6759,7 @@
         <v>2</v>
       </c>
       <c r="D122">
-        <f t="shared" si="28"/>
+        <f t="shared" si="27"/>
         <v>114451.25872361983</v>
       </c>
       <c r="E122">
@@ -6798,7 +6796,7 @@
         <v>0</v>
       </c>
       <c r="P122">
-        <f t="shared" si="29"/>
+        <f t="shared" si="28"/>
         <v>235010.93054261635</v>
       </c>
       <c r="Q122">
@@ -6825,7 +6823,7 @@
         <v>2</v>
       </c>
       <c r="D123">
-        <f t="shared" si="28"/>
+        <f t="shared" si="27"/>
         <v>114787.7594081375</v>
       </c>
       <c r="E123">
@@ -6862,7 +6860,7 @@
         <v>0</v>
       </c>
       <c r="P123">
-        <f t="shared" si="29"/>
+        <f t="shared" si="28"/>
         <v>235347.43122713402</v>
       </c>
       <c r="Q123">

</xml_diff>

<commit_message>
Updating the validation plots and naming
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -817,7 +817,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -992,12 +992,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="35">
@@ -1408,10 +1402,10 @@
     <xf numFmtId="0" fontId="18" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3403,11 +3397,11 @@
       </c>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A33" s="26" t="s">
+      <c r="A33" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="26"/>
-      <c r="C33" s="26"/>
+      <c r="B33" s="27"/>
+      <c r="C33" s="27"/>
       <c r="D33">
         <f>D31-D32</f>
         <v>-785.66289527932531</v>
@@ -4610,11 +4604,11 @@
       </c>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A64" s="26" t="s">
+      <c r="A64" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="B64" s="26"/>
-      <c r="C64" s="26"/>
+      <c r="B64" s="27"/>
+      <c r="C64" s="27"/>
       <c r="D64" s="10">
         <f>D63-D62</f>
         <v>486.66028698880109</v>
@@ -4705,11 +4699,11 @@
       <c r="D66" s="13"/>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A67" s="26" t="s">
+      <c r="A67" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="B67" s="26"/>
-      <c r="C67" s="26"/>
+      <c r="B67" s="27"/>
+      <c r="C67" s="27"/>
       <c r="D67" s="10"/>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.4">
@@ -4783,10 +4777,10 @@
       </c>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A69" s="26" t="s">
+      <c r="A69" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="B69" s="26"/>
+      <c r="B69" s="27"/>
       <c r="C69" s="9"/>
       <c r="D69" s="10">
         <f>D68-D62</f>
@@ -5245,7 +5239,7 @@
       </c>
     </row>
     <row r="81" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A81" s="27"/>
+      <c r="A81" s="26"/>
       <c r="B81" s="2"/>
     </row>
     <row r="82" spans="1:22" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
Preventing plant shutdowns for 9000AF result
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A09BA11-C389-447D-B5FD-2BEDC67CF040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4676490A-5EA2-4847-AD16-7685D1A84BB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-94" yWindow="-94" windowWidth="33103" windowHeight="17983" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -54,6 +54,7 @@
     <author>tc={7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}</author>
     <author>tc={B7EDEAAD-67C9-4693-A0FC-570282E02182}</author>
     <author>tc={0EBBD83F-AB64-4248-87E6-B99F88EE5F88}</author>
+    <author>tc={4F558AE1-FE55-497E-AC12-603E221B46D5}</author>
     <author>tc={8E704477-0437-40A7-B175-85F6EA0FB52A}</author>
     <author>tc={9BC5A461-E691-49A7-9AA5-314B7AD6B728}</author>
     <author>tc={FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}</author>
@@ -197,7 +198,15 @@
     Only one plant shutdown allowed</t>
       </text>
     </comment>
-    <comment ref="A68" authorId="16" shapeId="0" xr:uid="{8E704477-0437-40A7-B175-85F6EA0FB52A}">
+    <comment ref="A66" authorId="16" shapeId="0" xr:uid="{4F558AE1-FE55-497E-AC12-603E221B46D5}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Specifically 725 kW, which is the peak power for the optimal full flex solution</t>
+      </text>
+    </comment>
+    <comment ref="A70" authorId="17" shapeId="0" xr:uid="{8E704477-0437-40A7-B175-85F6EA0FB52A}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -205,7 +214,7 @@
     Including this as the final result</t>
       </text>
     </comment>
-    <comment ref="L69" authorId="17" shapeId="0" xr:uid="{9BC5A461-E691-49A7-9AA5-314B7AD6B728}">
+    <comment ref="L71" authorId="18" shapeId="0" xr:uid="{9BC5A461-E691-49A7-9AA5-314B7AD6B728}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -213,7 +222,7 @@
     Just some random lower recovery periods</t>
       </text>
     </comment>
-    <comment ref="A76" authorId="18" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
+    <comment ref="A78" authorId="19" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -222,7 +231,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="A78" authorId="19" shapeId="0" xr:uid="{72AFD5EA-5AA9-4CD2-944C-D32BC94D67D2}">
+    <comment ref="A80" authorId="20" shapeId="0" xr:uid="{72AFD5EA-5AA9-4CD2-944C-D32BC94D67D2}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -230,7 +239,7 @@
     If RED, result is using the 2026 rate, but I’m updating to the 2023 version</t>
       </text>
     </comment>
-    <comment ref="A83" authorId="20" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
+    <comment ref="A85" authorId="21" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -238,7 +247,7 @@
     Pretty sure this solution is wrong, but I don’t think I need this case for the paper</t>
       </text>
     </comment>
-    <comment ref="A89" authorId="21" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A91" authorId="22" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -246,7 +255,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="A101" authorId="22" shapeId="0" xr:uid="{3B63C6BF-9DE1-4172-A721-F97EE0406603}">
+    <comment ref="A103" authorId="23" shapeId="0" xr:uid="{3B63C6BF-9DE1-4172-A721-F97EE0406603}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -254,7 +263,7 @@
     2.5x higher brine costs (1.08$/m3)</t>
       </text>
     </comment>
-    <comment ref="A104" authorId="23" shapeId="0" xr:uid="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
+    <comment ref="A106" authorId="24" shapeId="0" xr:uid="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -262,7 +271,7 @@
     5x brine costs (2.15 $/m3)</t>
       </text>
     </comment>
-    <comment ref="A107" authorId="24" shapeId="0" xr:uid="{9D93D39A-4E12-4E91-8443-F39D5B5EA779}">
+    <comment ref="A109" authorId="25" shapeId="0" xr:uid="{9D93D39A-4E12-4E91-8443-F39D5B5EA779}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -270,7 +279,7 @@
     Working Hours = 8 AM to 5 PM</t>
       </text>
     </comment>
-    <comment ref="A112" authorId="25" shapeId="0" xr:uid="{9585276E-E9B8-4AFF-9F58-E3ADC73D024E}">
+    <comment ref="A114" authorId="26" shapeId="0" xr:uid="{9585276E-E9B8-4AFF-9F58-E3ADC73D024E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -278,7 +287,7 @@
     Five Shutdowns</t>
       </text>
     </comment>
-    <comment ref="T120" authorId="26" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T122" authorId="27" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -497,7 +506,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="104">
   <si>
     <t>Season</t>
   </si>
@@ -806,6 +815,9 @@
   </si>
   <si>
     <t>FOUR TRAINS</t>
+  </si>
+  <si>
+    <t>Result with a lower baseline peak power</t>
   </si>
 </sst>
 </file>
@@ -817,7 +829,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -992,6 +1004,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="35">
@@ -1838,38 +1856,41 @@
   <threadedComment ref="A63" dT="2026-07-22T21:09:49.14" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{0EBBD83F-AB64-4248-87E6-B99F88EE5F88}">
     <text>Only one plant shutdown allowed</text>
   </threadedComment>
-  <threadedComment ref="A68" dT="2026-08-03T21:10:04.14" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{8E704477-0437-40A7-B175-85F6EA0FB52A}">
+  <threadedComment ref="A66" dT="2026-09-15T16:14:38.89" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4F558AE1-FE55-497E-AC12-603E221B46D5}">
+    <text>Specifically 725 kW, which is the peak power for the optimal full flex solution</text>
+  </threadedComment>
+  <threadedComment ref="A70" dT="2026-08-03T21:10:04.14" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{8E704477-0437-40A7-B175-85F6EA0FB52A}">
     <text>Including this as the final result</text>
   </threadedComment>
-  <threadedComment ref="L69" dT="2026-08-03T21:09:16.86" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9BC5A461-E691-49A7-9AA5-314B7AD6B728}">
+  <threadedComment ref="L71" dT="2026-08-03T21:09:16.86" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9BC5A461-E691-49A7-9AA5-314B7AD6B728}">
     <text>Just some random lower recovery periods</text>
   </threadedComment>
-  <threadedComment ref="A76" dT="2026-07-22T16:56:30.58" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
+  <threadedComment ref="A78" dT="2026-07-22T16:56:30.58" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
     <text xml:space="preserve">This should be the same as the other DR solution, except for the demand response revenue
 </text>
   </threadedComment>
-  <threadedComment ref="A78" dT="2026-09-11T22:19:30.96" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{72AFD5EA-5AA9-4CD2-944C-D32BC94D67D2}">
+  <threadedComment ref="A80" dT="2026-09-11T22:19:30.96" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{72AFD5EA-5AA9-4CD2-944C-D32BC94D67D2}">
     <text>If RED, result is using the 2026 rate, but I’m updating to the 2023 version</text>
   </threadedComment>
-  <threadedComment ref="A83" dT="2026-07-21T19:23:55.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4644E393-F522-4E79-88BA-041770B595A7}">
+  <threadedComment ref="A85" dT="2026-07-21T19:23:55.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4644E393-F522-4E79-88BA-041770B595A7}">
     <text>Pretty sure this solution is wrong, but I don’t think I need this case for the paper</text>
   </threadedComment>
-  <threadedComment ref="A89" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+  <threadedComment ref="A91" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
     <text>The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</text>
   </threadedComment>
-  <threadedComment ref="A101" dT="2026-08-09T17:04:16.49" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{3B63C6BF-9DE1-4172-A721-F97EE0406603}">
+  <threadedComment ref="A103" dT="2026-08-09T17:04:16.49" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{3B63C6BF-9DE1-4172-A721-F97EE0406603}">
     <text>2.5x higher brine costs (1.08$/m3)</text>
   </threadedComment>
-  <threadedComment ref="A104" dT="2026-08-09T17:05:17.32" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
+  <threadedComment ref="A106" dT="2026-08-09T17:05:17.32" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
     <text>5x brine costs (2.15 $/m3)</text>
   </threadedComment>
-  <threadedComment ref="A107" dT="2026-08-18T21:09:34.88" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9D93D39A-4E12-4E91-8443-F39D5B5EA779}">
+  <threadedComment ref="A109" dT="2026-08-18T21:09:34.88" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9D93D39A-4E12-4E91-8443-F39D5B5EA779}">
     <text>Working Hours = 8 AM to 5 PM</text>
   </threadedComment>
-  <threadedComment ref="A112" dT="2026-08-28T19:35:29.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9585276E-E9B8-4AFF-9F58-E3ADC73D024E}">
+  <threadedComment ref="A114" dT="2026-08-28T19:35:29.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9585276E-E9B8-4AFF-9F58-E3ADC73D024E}">
     <text>Five Shutdowns</text>
   </threadedComment>
-  <threadedComment ref="T120" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="T122" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1964,7 +1985,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:V123"/>
+  <dimension ref="A1:V125"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="9.61328125" customWidth="1"/>
@@ -4693,1271 +4714,1273 @@
       <c r="D65" s="10"/>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A66" s="9"/>
-      <c r="B66" s="9"/>
-      <c r="C66" s="9"/>
-      <c r="D66" s="13"/>
+      <c r="A66" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="B66" s="27"/>
+      <c r="C66" s="27"/>
+      <c r="D66" s="27"/>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A67" s="27" t="s">
-        <v>60</v>
-      </c>
-      <c r="B67" s="27"/>
-      <c r="C67" s="27"/>
-      <c r="D67" s="10"/>
+      <c r="A67" t="s">
+        <v>22</v>
+      </c>
+      <c r="B67" t="s">
+        <v>21</v>
+      </c>
+      <c r="C67">
+        <v>4</v>
+      </c>
+      <c r="D67" s="10">
+        <f>J67+K67+L67+M67+N67-O67</f>
+        <v>111404.48735261035</v>
+      </c>
+      <c r="E67">
+        <v>282179.67210423102</v>
+      </c>
+      <c r="F67">
+        <v>0.82037834333814497</v>
+      </c>
+      <c r="G67">
+        <v>19838.6932313</v>
+      </c>
+      <c r="H67">
+        <v>6386.10618344667</v>
+      </c>
+      <c r="I67" s="8">
+        <v>9.2973424231475194E-6</v>
+      </c>
+      <c r="J67">
+        <v>26224.799424043998</v>
+      </c>
+      <c r="K67">
+        <v>50899.945350741502</v>
+      </c>
+      <c r="L67">
+        <v>20114.677460726201</v>
+      </c>
+      <c r="M67">
+        <v>19952.6871621766</v>
+      </c>
+      <c r="N67">
+        <v>1462.3779549220301</v>
+      </c>
+      <c r="O67">
+        <v>7250</v>
+      </c>
+      <c r="P67">
+        <f t="shared" ref="P67" si="14">D67+$P$1</f>
+        <v>231964.15917160688</v>
+      </c>
+      <c r="Q67">
+        <v>1426.8142686552001</v>
+      </c>
+      <c r="R67">
+        <v>20405.960832041099</v>
+      </c>
+      <c r="S67">
+        <v>566.83224533447503</v>
+      </c>
+      <c r="T67">
+        <v>0.42602809634619399</v>
+      </c>
+      <c r="U67">
+        <v>88484.431706385905</v>
+      </c>
+      <c r="V67">
+        <v>670.33660383625704</v>
+      </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A68" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B68" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C68">
-        <v>4</v>
-      </c>
-      <c r="D68">
-        <f>J68+K68+L68+M68+N68-O68</f>
-        <v>107688.42172332953</v>
-      </c>
-      <c r="E68">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F68">
-        <v>0.80720919866445495</v>
-      </c>
-      <c r="G68" s="10">
-        <v>19953.454987134999</v>
-      </c>
-      <c r="H68" s="10">
-        <v>6500.5540138059996</v>
-      </c>
-      <c r="I68" s="10">
-        <v>1.4041882744936899E-5</v>
-      </c>
-      <c r="J68" s="10">
-        <v>26454.009014982901</v>
-      </c>
-      <c r="K68" s="10">
-        <v>50854.945205479497</v>
-      </c>
-      <c r="L68" s="10">
-        <v>19993.739942922399</v>
-      </c>
-      <c r="M68" s="10">
-        <v>19943.3496050227</v>
-      </c>
-      <c r="N68" s="10">
-        <v>1462.3779549220301</v>
-      </c>
-      <c r="O68">
-        <v>11020</v>
-      </c>
-      <c r="P68">
-        <f t="shared" ref="P68" si="14">D68+$P$1</f>
-        <v>228248.09354232607</v>
-      </c>
-      <c r="Q68">
-        <v>1452.3847453508599</v>
-      </c>
-      <c r="R68">
-        <v>38020.577577602002</v>
-      </c>
-      <c r="S68">
-        <v>884.19947854888403</v>
-      </c>
-      <c r="T68">
-        <v>0.32639110364227297</v>
-      </c>
-      <c r="U68">
-        <v>43796.182548819299</v>
-      </c>
-      <c r="V68">
-        <v>350.36946039055402</v>
-      </c>
+      <c r="A68" s="9"/>
+      <c r="B68" s="9"/>
+      <c r="C68" s="9"/>
+      <c r="D68" s="13"/>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A69" s="27" t="s">
+        <v>60</v>
+      </c>
+      <c r="B69" s="27"/>
+      <c r="C69" s="27"/>
+      <c r="D69" s="10"/>
+    </row>
+    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A70" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B70" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C70">
+        <v>4</v>
+      </c>
+      <c r="D70">
+        <f>J70+K70+L70+M70+N70-O70</f>
+        <v>107688.42172332953</v>
+      </c>
+      <c r="E70">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F70">
+        <v>0.80720919866445495</v>
+      </c>
+      <c r="G70" s="10">
+        <v>19953.454987134999</v>
+      </c>
+      <c r="H70" s="10">
+        <v>6500.5540138059996</v>
+      </c>
+      <c r="I70" s="10">
+        <v>1.4041882744936899E-5</v>
+      </c>
+      <c r="J70" s="10">
+        <v>26454.009014982901</v>
+      </c>
+      <c r="K70" s="10">
+        <v>50854.945205479497</v>
+      </c>
+      <c r="L70" s="10">
+        <v>19993.739942922399</v>
+      </c>
+      <c r="M70" s="10">
+        <v>19943.3496050227</v>
+      </c>
+      <c r="N70" s="10">
+        <v>1462.3779549220301</v>
+      </c>
+      <c r="O70">
+        <v>11020</v>
+      </c>
+      <c r="P70">
+        <f t="shared" ref="P70" si="15">D70+$P$1</f>
+        <v>228248.09354232607</v>
+      </c>
+      <c r="Q70">
+        <v>1452.3847453508599</v>
+      </c>
+      <c r="R70">
+        <v>38020.577577602002</v>
+      </c>
+      <c r="S70">
+        <v>884.19947854888403</v>
+      </c>
+      <c r="T70">
+        <v>0.32639110364227297</v>
+      </c>
+      <c r="U70">
+        <v>43796.182548819299</v>
+      </c>
+      <c r="V70">
+        <v>350.36946039055402</v>
+      </c>
+    </row>
+    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A71" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="B69" s="27"/>
-      <c r="C69" s="9"/>
-      <c r="D69" s="10">
-        <f>D68-D62</f>
+      <c r="B71" s="27"/>
+      <c r="C71" s="9"/>
+      <c r="D71" s="10">
+        <f>D70-D62</f>
         <v>133.12347700698592</v>
       </c>
-      <c r="E69" s="10">
-        <f t="shared" ref="E69:P69" si="15">E68-E62</f>
-        <v>0</v>
-      </c>
-      <c r="F69" s="10">
-        <f t="shared" si="15"/>
+      <c r="E71" s="10">
+        <f t="shared" ref="E71:P71" si="16">E70-E62</f>
+        <v>0</v>
+      </c>
+      <c r="F71" s="10">
+        <f t="shared" si="16"/>
         <v>4.7176848858698772E-4</v>
       </c>
-      <c r="G69" s="10">
-        <f t="shared" si="15"/>
+      <c r="G71" s="10">
+        <f t="shared" si="16"/>
         <v>336.18543171020065</v>
       </c>
-      <c r="H69" s="10">
-        <f t="shared" si="15"/>
+      <c r="H71" s="10">
+        <f t="shared" si="16"/>
         <v>322.76314238460964</v>
       </c>
-      <c r="I69" s="10">
-        <f t="shared" si="15"/>
+      <c r="I71" s="10">
+        <f t="shared" si="16"/>
         <v>-8.5546091703980134E-7</v>
       </c>
-      <c r="J69" s="10">
-        <f t="shared" si="15"/>
+      <c r="J71" s="10">
+        <f t="shared" si="16"/>
         <v>658.94857323930046</v>
       </c>
-      <c r="K69" s="10">
-        <f t="shared" si="15"/>
+      <c r="K71" s="10">
+        <f t="shared" si="16"/>
         <v>-135.00002418200165</v>
       </c>
-      <c r="L69" s="10">
-        <f t="shared" si="15"/>
+      <c r="L71" s="10">
+        <f t="shared" si="16"/>
         <v>-362.81256703230247</v>
       </c>
-      <c r="M69" s="10">
-        <f t="shared" si="15"/>
+      <c r="M71" s="10">
+        <f t="shared" si="16"/>
         <v>-28.012505017999501</v>
       </c>
-      <c r="N69" s="10">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-      <c r="O69" s="10">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-      <c r="P69" s="10">
-        <f t="shared" si="15"/>
+      <c r="N71" s="10">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="O71" s="10">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="P71" s="10">
+        <f t="shared" si="16"/>
         <v>133.12347700700047</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A70" s="9"/>
-      <c r="B70" s="9"/>
-      <c r="C70" s="9"/>
-      <c r="D70" s="10"/>
-      <c r="E70" s="10"/>
-      <c r="F70" s="10"/>
-      <c r="G70" s="10"/>
-      <c r="H70" s="10"/>
-      <c r="I70" s="10"/>
-      <c r="J70" s="10"/>
-      <c r="K70" s="10">
-        <f>K68+L68+M68-K5</f>
+    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A72" s="9"/>
+      <c r="B72" s="9"/>
+      <c r="C72" s="9"/>
+      <c r="D72" s="10"/>
+      <c r="E72" s="10"/>
+      <c r="F72" s="10"/>
+      <c r="G72" s="10"/>
+      <c r="H72" s="10"/>
+      <c r="I72" s="10"/>
+      <c r="J72" s="10"/>
+      <c r="K72" s="10">
+        <f>K70+L70+M70-K5</f>
         <v>5347.5218722698046</v>
       </c>
-      <c r="L70" s="10"/>
-      <c r="M70" s="10"/>
-      <c r="N70" s="10"/>
-      <c r="O70" s="10"/>
-      <c r="P70" s="10"/>
-    </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A71" s="1" t="s">
+      <c r="L72" s="10"/>
+      <c r="M72" s="10"/>
+      <c r="N72" s="10"/>
+      <c r="O72" s="10"/>
+      <c r="P72" s="10"/>
+    </row>
+    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A73" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G71" s="4"/>
-    </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A72" s="3" t="s">
+      <c r="G73" s="4"/>
+    </row>
+    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A74" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B72" s="3" t="s">
+      <c r="B74" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C72" s="3">
-        <v>0</v>
-      </c>
-      <c r="G72" s="4"/>
-    </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A73" t="s">
+      <c r="C74" s="3">
+        <v>0</v>
+      </c>
+      <c r="G74" s="4"/>
+    </row>
+    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A75" t="s">
         <v>22</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B75" t="s">
         <v>23</v>
       </c>
-      <c r="C73">
-        <v>0</v>
-      </c>
-      <c r="D73">
-        <f>J73+K73+L73+M73+N73-O73</f>
+      <c r="C75">
+        <v>0</v>
+      </c>
+      <c r="D75">
+        <f>J75+K75+L75+M75+N75-O75</f>
         <v>125093.23428318274</v>
       </c>
-      <c r="E73">
+      <c r="E75">
         <v>282190.859999999</v>
       </c>
-      <c r="F73">
+      <c r="F75">
         <v>0.86904083066499505</v>
       </c>
-      <c r="G73" s="10">
+      <c r="G75" s="10">
         <v>24203.497764766002</v>
       </c>
-      <c r="H73" s="10">
+      <c r="H75" s="10">
         <v>4932.7238161263904</v>
       </c>
-      <c r="I73" s="10">
+      <c r="I75" s="10">
         <v>9098.5748223234004</v>
       </c>
-      <c r="J73" s="10">
+      <c r="J75" s="10">
         <v>38234.796403215798</v>
       </c>
-      <c r="K73" s="10">
+      <c r="K75" s="10">
         <v>50845.200000000099</v>
       </c>
-      <c r="L73" s="10">
+      <c r="L75" s="10">
         <v>15304.405199999899</v>
       </c>
-      <c r="M73" s="10">
+      <c r="M75" s="10">
         <v>19298.29566</v>
       </c>
-      <c r="N73" s="10">
+      <c r="N75" s="10">
         <v>1409.83742959549</v>
       </c>
-      <c r="O73">
+      <c r="O75">
         <v>-0.69959037146548997</v>
       </c>
-      <c r="P73">
-        <f>D73+$P$1</f>
+      <c r="P75">
+        <f>D75+$P$1</f>
         <v>245652.90610217926</v>
       </c>
-      <c r="Q73">
+      <c r="Q75">
         <v>1102.0926609763501</v>
       </c>
-      <c r="R73">
-        <v>0</v>
-      </c>
-      <c r="U73">
+      <c r="R75">
+        <v>0</v>
+      </c>
+      <c r="U75">
         <v>15.5670440273115</v>
       </c>
-      <c r="V73">
+      <c r="V75">
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A74" s="3"/>
-      <c r="B74" s="3"/>
-      <c r="C74" s="3"/>
-      <c r="G74" s="4"/>
-    </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A75" s="3" t="s">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A76" s="3"/>
+      <c r="B76" s="3"/>
+      <c r="C76" s="3"/>
+      <c r="G76" s="4"/>
+    </row>
+    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A77" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B75" s="3" t="s">
+      <c r="B77" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C75" s="3">
+      <c r="C77" s="3">
         <v>4</v>
       </c>
-      <c r="G75" s="4"/>
-    </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A76" t="s">
+      <c r="G77" s="4"/>
+    </row>
+    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A78" t="s">
         <v>22</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B78" t="s">
         <v>21</v>
       </c>
-      <c r="C76">
+      <c r="C78">
         <v>4</v>
       </c>
-      <c r="D76">
-        <f>J76+K76+L76+M76+N76-O76</f>
+      <c r="D78">
+        <f>J78+K78+L78+M78+N78-O78</f>
         <v>110388.32172332953</v>
       </c>
-      <c r="E76">
+      <c r="E78">
         <v>282179.67123287602</v>
       </c>
-      <c r="F76">
+      <c r="F78">
         <v>0.80720919866445495</v>
       </c>
-      <c r="G76" s="10">
+      <c r="G78" s="10">
         <v>19953.454987134999</v>
       </c>
-      <c r="H76" s="10">
+      <c r="H78" s="10">
         <v>6500.5540138059996</v>
       </c>
-      <c r="I76" s="10">
+      <c r="I78" s="10">
         <v>1.4041882744936899E-5</v>
       </c>
-      <c r="J76" s="10">
+      <c r="J78" s="10">
         <v>26454.009014982901</v>
       </c>
-      <c r="K76" s="10">
+      <c r="K78" s="10">
         <v>50854.945205479497</v>
       </c>
-      <c r="L76" s="10">
+      <c r="L78" s="10">
         <v>19993.739942922399</v>
       </c>
-      <c r="M76" s="10">
+      <c r="M78" s="10">
         <v>19943.3496050227</v>
       </c>
-      <c r="N76" s="10">
+      <c r="N78" s="10">
         <v>1462.3779549220301</v>
       </c>
-      <c r="O76">
+      <c r="O78">
         <v>8320.1</v>
       </c>
-      <c r="P76">
+      <c r="P78">
         <v>230384.72273471201</v>
       </c>
-      <c r="Q76">
+      <c r="Q78">
         <v>1403.49453592792</v>
       </c>
-      <c r="R76">
+      <c r="R78">
         <v>34518.506961381201</v>
       </c>
-      <c r="S76">
+      <c r="S78">
         <v>841.91480393612801</v>
       </c>
-      <c r="T76">
+      <c r="T78">
         <v>0.38784649209264499</v>
       </c>
-      <c r="U76">
+      <c r="U78">
         <v>38264.627438579002</v>
       </c>
-      <c r="V76">
+      <c r="V78">
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A77" s="5"/>
-      <c r="B77" s="5"/>
-      <c r="D77">
-        <f>D76-D73</f>
+    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A79" s="5"/>
+      <c r="B79" s="5"/>
+      <c r="D79">
+        <f>D78-D75</f>
         <v>-14704.912559853212</v>
       </c>
-      <c r="E77">
-        <f t="shared" ref="E77:V77" si="16">E76-E73</f>
+      <c r="E79">
+        <f t="shared" ref="E79:V79" si="17">E78-E75</f>
         <v>-11.188767122977879</v>
       </c>
-      <c r="F77">
-        <f t="shared" si="16"/>
+      <c r="F79">
+        <f t="shared" si="17"/>
         <v>-6.1831632000540093E-2</v>
       </c>
-      <c r="G77">
-        <f t="shared" si="16"/>
+      <c r="G79">
+        <f t="shared" si="17"/>
         <v>-4250.0427776310025</v>
       </c>
-      <c r="H77">
-        <f t="shared" si="16"/>
+      <c r="H79">
+        <f t="shared" si="17"/>
         <v>1567.8301976796092</v>
       </c>
-      <c r="I77">
-        <f t="shared" si="16"/>
+      <c r="I79">
+        <f t="shared" si="17"/>
         <v>-9098.5748082815171</v>
       </c>
-      <c r="J77">
-        <f t="shared" si="16"/>
+      <c r="J79">
+        <f t="shared" si="17"/>
         <v>-11780.787388232897</v>
       </c>
-      <c r="K77">
-        <f t="shared" si="16"/>
+      <c r="K79">
+        <f t="shared" si="17"/>
         <v>9.7452054793975549</v>
       </c>
-      <c r="L77">
-        <f t="shared" si="16"/>
+      <c r="L79">
+        <f t="shared" si="17"/>
         <v>4689.3347429224996</v>
       </c>
-      <c r="M77">
-        <f t="shared" si="16"/>
+      <c r="M79">
+        <f t="shared" si="17"/>
         <v>645.05394502270065</v>
       </c>
-      <c r="N77">
-        <f t="shared" si="16"/>
+      <c r="N79">
+        <f t="shared" si="17"/>
         <v>52.540525326540092</v>
       </c>
-      <c r="O77">
-        <f t="shared" si="16"/>
+      <c r="O79">
+        <f t="shared" si="17"/>
         <v>8320.7995903714655</v>
       </c>
-      <c r="P77">
-        <f t="shared" si="16"/>
+      <c r="P79">
+        <f t="shared" si="17"/>
         <v>-15268.183367467253</v>
       </c>
-      <c r="Q77">
-        <f t="shared" si="16"/>
+      <c r="Q79">
+        <f t="shared" si="17"/>
         <v>301.40187495156988</v>
       </c>
-      <c r="R77">
-        <f t="shared" si="16"/>
+      <c r="R79">
+        <f t="shared" si="17"/>
         <v>34518.506961381201</v>
       </c>
-      <c r="S77">
-        <f t="shared" si="16"/>
+      <c r="S79">
+        <f t="shared" si="17"/>
         <v>841.91480393612801</v>
       </c>
-      <c r="T77">
-        <f t="shared" si="16"/>
+      <c r="T79">
+        <f t="shared" si="17"/>
         <v>0.38784649209264499</v>
       </c>
-      <c r="U77">
-        <f t="shared" si="16"/>
+      <c r="U79">
+        <f t="shared" si="17"/>
         <v>38249.060394551692</v>
       </c>
-      <c r="V77">
-        <f t="shared" si="16"/>
+      <c r="V79">
+        <f t="shared" si="17"/>
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A78" s="1" t="s">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A80" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A79" s="2" t="s">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A81" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="B81" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C79">
-        <v>0</v>
-      </c>
-      <c r="D79">
-        <f>J79+K79+L79+M79+N79</f>
+      <c r="C81">
+        <v>0</v>
+      </c>
+      <c r="D81">
+        <f>J81+K81+L81+M81+N81</f>
         <v>116023.2890300647</v>
       </c>
-      <c r="E79">
+      <c r="E81">
         <v>282179.67123287602</v>
       </c>
-      <c r="F79">
+      <c r="F81">
         <v>0.83841249022441</v>
       </c>
-      <c r="G79">
+      <c r="G81">
         <v>20114.092712805999</v>
       </c>
-      <c r="H79">
+      <c r="H81">
         <v>6942.2846600808298</v>
       </c>
-      <c r="I79">
+      <c r="I81">
         <v>2530.0880681377598</v>
       </c>
-      <c r="J79">
+      <c r="J81">
         <v>29586.4654410246</v>
       </c>
-      <c r="K79">
+      <c r="K81">
         <v>50843.184005923598</v>
       </c>
-      <c r="L79">
+      <c r="L81">
         <v>15303.798385783</v>
       </c>
-      <c r="M79">
+      <c r="M81">
         <v>19297.5304894482</v>
       </c>
-      <c r="N79">
+      <c r="N81">
         <v>992.31070788530405</v>
       </c>
-      <c r="O79">
-        <v>0</v>
-      </c>
-      <c r="P79">
-        <f t="shared" ref="P79:P80" si="17">D79+$P$1</f>
+      <c r="O81">
+        <v>0</v>
+      </c>
+      <c r="P81">
+        <f t="shared" ref="P81:P82" si="18">D81+$P$1</f>
         <v>236582.9608490612</v>
       </c>
-      <c r="Q79">
+      <c r="Q81">
         <v>1101.8347602124099</v>
       </c>
-      <c r="R79">
-        <v>0</v>
-      </c>
-      <c r="S79">
-        <v>0</v>
-      </c>
-      <c r="T79">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A80" s="5" t="s">
+      <c r="R81">
+        <v>0</v>
+      </c>
+      <c r="S81">
+        <v>0</v>
+      </c>
+      <c r="T81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A82" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B80" s="5" t="s">
+      <c r="B82" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C80">
-        <v>0</v>
-      </c>
-      <c r="D80">
-        <f>J80+K80+L80+M80+N80</f>
-        <v>124337.62912011228</v>
-      </c>
-      <c r="E80">
-        <v>282190.859999999</v>
-      </c>
-      <c r="F80">
-        <v>0.86636319198077105</v>
-      </c>
-      <c r="G80">
-        <v>22795.571059233</v>
-      </c>
-      <c r="H80">
-        <v>5233.0127982051599</v>
-      </c>
-      <c r="I80">
-        <v>9451.3069638763409</v>
-      </c>
-      <c r="J80">
-        <v>37479.890821314497</v>
-      </c>
-      <c r="K80">
-        <v>50845.200002362697</v>
-      </c>
-      <c r="L80">
-        <v>15304.4052063494</v>
-      </c>
-      <c r="M80">
-        <v>19298.295660490199</v>
-      </c>
-      <c r="N80">
-        <v>1409.83742959549</v>
-      </c>
-      <c r="O80">
-        <v>0</v>
-      </c>
-      <c r="P80">
-        <f t="shared" si="17"/>
-        <v>244897.3009391088</v>
-      </c>
-      <c r="Q80">
-        <v>1127.3472943468801</v>
-      </c>
-      <c r="R80">
-        <v>0</v>
-      </c>
-      <c r="S80">
-        <v>0</v>
-      </c>
-      <c r="T80">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A81" s="26"/>
-      <c r="B81" s="2"/>
-    </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A82" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>21</v>
-      </c>
       <c r="C82">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D82">
         <f>J82+K82+L82+M82+N82</f>
+        <v>124337.62912011228</v>
+      </c>
+      <c r="E82">
+        <v>282190.859999999</v>
+      </c>
+      <c r="F82">
+        <v>0.86636319198077105</v>
+      </c>
+      <c r="G82">
+        <v>22795.571059233</v>
+      </c>
+      <c r="H82">
+        <v>5233.0127982051599</v>
+      </c>
+      <c r="I82">
+        <v>9451.3069638763409</v>
+      </c>
+      <c r="J82">
+        <v>37479.890821314497</v>
+      </c>
+      <c r="K82">
+        <v>50845.200002362697</v>
+      </c>
+      <c r="L82">
+        <v>15304.4052063494</v>
+      </c>
+      <c r="M82">
+        <v>19298.295660490199</v>
+      </c>
+      <c r="N82">
+        <v>1409.83742959549</v>
+      </c>
+      <c r="O82">
+        <v>0</v>
+      </c>
+      <c r="P82">
+        <f t="shared" si="18"/>
+        <v>244897.3009391088</v>
+      </c>
+      <c r="Q82">
+        <v>1127.3472943468801</v>
+      </c>
+      <c r="R82">
+        <v>0</v>
+      </c>
+      <c r="S82">
+        <v>0</v>
+      </c>
+      <c r="T82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A83" s="26"/>
+      <c r="B83" s="2"/>
+    </row>
+    <row r="84" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A84" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C84">
+        <v>2</v>
+      </c>
+      <c r="D84">
+        <f>J84+K84+L84+M84+N84</f>
         <v>116706.4157905087</v>
       </c>
-      <c r="E82">
+      <c r="E84">
         <v>282179.67125387199</v>
       </c>
-      <c r="F82">
+      <c r="F84">
         <v>0.840833383054163</v>
       </c>
-      <c r="G82" s="4">
+      <c r="G84" s="4">
         <v>20578.507216446698</v>
       </c>
-      <c r="H82">
+      <c r="H84">
         <v>7102.57515066207</v>
       </c>
-      <c r="I82">
+      <c r="I84">
         <v>2588.5052959285099</v>
       </c>
-      <c r="J82">
+      <c r="J84">
         <v>30269.587663037299</v>
       </c>
-      <c r="K82">
+      <c r="K84">
         <v>50843.185173268597</v>
       </c>
-      <c r="L82">
+      <c r="L84">
         <v>15303.8015139941</v>
       </c>
-      <c r="M82">
+      <c r="M84">
         <v>19297.530732323401</v>
       </c>
-      <c r="N82">
+      <c r="N84">
         <v>992.31070788530405</v>
       </c>
-      <c r="O82">
-        <v>0</v>
-      </c>
-      <c r="P82">
-        <f t="shared" ref="P82:P83" si="18">D82+$P$1</f>
+      <c r="O84">
+        <v>0</v>
+      </c>
+      <c r="P84">
+        <f t="shared" ref="P84:P85" si="19">D84+$P$1</f>
         <v>237266.08760950522</v>
       </c>
-      <c r="Q82">
+      <c r="Q84">
         <v>1127.2750356983099</v>
       </c>
-      <c r="R82">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A83" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C83">
-        <v>2</v>
-      </c>
-      <c r="D83">
-        <f>J83+K83+L83+M83+N83</f>
-        <v>121633.35860365373</v>
-      </c>
-      <c r="E83">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F83">
-        <v>0.85824890324911396</v>
-      </c>
-      <c r="G83" s="4">
-        <v>20824.7129679639</v>
-      </c>
-      <c r="H83">
-        <v>7456.39074483072</v>
-      </c>
-      <c r="I83">
-        <v>5114.4587365303096</v>
-      </c>
-      <c r="J83">
-        <v>33395.562449324898</v>
-      </c>
-      <c r="K83">
-        <v>51302.320205525801</v>
-      </c>
-      <c r="L83">
-        <v>16537.7269222135</v>
-      </c>
-      <c r="M83">
-        <v>19392.801250865799</v>
-      </c>
-      <c r="N83">
-        <v>1004.9477757237401</v>
-      </c>
-      <c r="O83">
-        <v>0</v>
-      </c>
-      <c r="P83">
-        <f t="shared" si="18"/>
-        <v>242193.03042265025</v>
-      </c>
-      <c r="Q83">
-        <v>1183.4303612998101</v>
-      </c>
-      <c r="R83">
-        <v>15931.1957490451</v>
-      </c>
-      <c r="S83">
-        <v>346.33034237054602</v>
-      </c>
-      <c r="T83">
-        <v>1.0959871186973</v>
-      </c>
-    </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A84" s="2"/>
-      <c r="B84" s="2"/>
+      <c r="R84">
+        <v>0</v>
+      </c>
     </row>
     <row r="85" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A85" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C85">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D85">
         <f>J85+K85+L85+M85+N85</f>
+        <v>121633.35860365373</v>
+      </c>
+      <c r="E85">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F85">
+        <v>0.85824890324911396</v>
+      </c>
+      <c r="G85" s="4">
+        <v>20824.7129679639</v>
+      </c>
+      <c r="H85">
+        <v>7456.39074483072</v>
+      </c>
+      <c r="I85">
+        <v>5114.4587365303096</v>
+      </c>
+      <c r="J85">
+        <v>33395.562449324898</v>
+      </c>
+      <c r="K85">
+        <v>51302.320205525801</v>
+      </c>
+      <c r="L85">
+        <v>16537.7269222135</v>
+      </c>
+      <c r="M85">
+        <v>19392.801250865799</v>
+      </c>
+      <c r="N85">
+        <v>1004.9477757237401</v>
+      </c>
+      <c r="O85">
+        <v>0</v>
+      </c>
+      <c r="P85">
+        <f t="shared" si="19"/>
+        <v>242193.03042265025</v>
+      </c>
+      <c r="Q85">
+        <v>1183.4303612998101</v>
+      </c>
+      <c r="R85">
+        <v>15931.1957490451</v>
+      </c>
+      <c r="S85">
+        <v>346.33034237054602</v>
+      </c>
+      <c r="T85">
+        <v>1.0959871186973</v>
+      </c>
+    </row>
+    <row r="86" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A86" s="2"/>
+      <c r="B86" s="2"/>
+    </row>
+    <row r="87" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A87" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C87">
+        <v>4</v>
+      </c>
+      <c r="D87">
+        <f>J87+K87+L87+M87+N87</f>
         <v>116706.4157905051</v>
       </c>
-      <c r="E85">
+      <c r="E87">
         <v>282179.671253876</v>
       </c>
-      <c r="F85">
+      <c r="F87">
         <v>0.84083338305413902</v>
       </c>
-      <c r="G85" s="4">
+      <c r="G87" s="4">
         <v>20578.5072164468</v>
       </c>
-      <c r="H85">
+      <c r="H87">
         <v>7102.5751506616798</v>
       </c>
-      <c r="I85">
+      <c r="I87">
         <v>2588.50529592865</v>
       </c>
-      <c r="J85">
+      <c r="J87">
         <v>30269.587663037099</v>
       </c>
-      <c r="K85">
+      <c r="K87">
         <v>50843.185173268197</v>
       </c>
-      <c r="L85">
+      <c r="L87">
         <v>15303.8015139912</v>
       </c>
-      <c r="M85">
+      <c r="M87">
         <v>19297.530732323299</v>
       </c>
-      <c r="N85">
+      <c r="N87">
         <v>992.31070788530405</v>
       </c>
-      <c r="O85">
-        <v>0</v>
-      </c>
-      <c r="P85">
-        <f t="shared" ref="P85:P89" si="19">D85+$P$1</f>
+      <c r="O87">
+        <v>0</v>
+      </c>
+      <c r="P87">
+        <f t="shared" ref="P87:P91" si="20">D87+$P$1</f>
         <v>237266.08760950161</v>
       </c>
-      <c r="Q85">
+      <c r="Q87">
         <v>1127.2750356983499</v>
       </c>
-      <c r="R85">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A86" s="5" t="s">
+      <c r="R87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A88" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B86" s="5" t="s">
+      <c r="B88" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C86">
+      <c r="C88">
         <v>4</v>
       </c>
-      <c r="D86">
-        <f>J86+K86+L86+M86+N86</f>
+      <c r="D88">
+        <f>J88+K88+L88+M88+N88</f>
         <v>119679.31713838593</v>
       </c>
-      <c r="E86">
+      <c r="E88">
         <v>282179.67123287602</v>
       </c>
-      <c r="F86">
+      <c r="F88">
         <v>0.84981637630953</v>
       </c>
-      <c r="G86">
+      <c r="G88">
         <v>21259.596722088401</v>
       </c>
-      <c r="H86">
+      <c r="H88">
         <v>5421.7142614628301</v>
       </c>
-      <c r="I86">
+      <c r="I88">
         <v>4952.1226155222203</v>
       </c>
-      <c r="J86">
+      <c r="J88">
         <v>31633.433599073502</v>
       </c>
-      <c r="K86">
+      <c r="K88">
         <v>51143.819864261903</v>
       </c>
-      <c r="L86">
+      <c r="L88">
         <v>16111.757255067099</v>
       </c>
-      <c r="M86">
+      <c r="M88">
         <v>19359.912430053599</v>
       </c>
-      <c r="N86">
+      <c r="N88">
         <v>1430.39398992981</v>
       </c>
-      <c r="O86">
-        <v>0</v>
-      </c>
-      <c r="P86">
-        <f t="shared" si="19"/>
+      <c r="O88">
+        <v>0</v>
+      </c>
+      <c r="P88">
+        <f t="shared" si="20"/>
         <v>240238.98895738245</v>
       </c>
-      <c r="Q86">
+      <c r="Q88">
         <v>1167.9992270377099</v>
       </c>
-      <c r="R86">
+      <c r="R88">
         <v>12796.980451596301</v>
       </c>
-      <c r="S86">
+      <c r="S88">
         <v>511.87921806385202</v>
       </c>
-      <c r="T86">
+      <c r="T88">
         <v>3.2717316651185699E-2</v>
       </c>
-      <c r="U86">
+      <c r="U88">
         <v>9062.6004208208706</v>
       </c>
-      <c r="V86">
+      <c r="V88">
         <v>63.374828117628397</v>
       </c>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="K87">
-        <f>K86+L86+M86-(K80+L80+M80)</f>
+    <row r="89" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="K89">
+        <f>K88+L88+M88-(K82+L82+M82)</f>
         <v>1167.588680180299</v>
       </c>
-      <c r="P87">
-        <f t="shared" si="19"/>
+      <c r="P89">
+        <f t="shared" si="20"/>
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A88" s="1" t="s">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A90" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G88" s="4"/>
-    </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A89" t="s">
+      <c r="G90" s="4"/>
+    </row>
+    <row r="91" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A91" t="s">
         <v>22</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B91" t="s">
         <v>21</v>
       </c>
-      <c r="C89">
+      <c r="C91">
         <v>4</v>
       </c>
-      <c r="D89">
-        <f>J89+K89+L89+M89+N89</f>
+      <c r="D91">
+        <f>J91+K91+L91+M91+N91</f>
         <v>147118.48206815872</v>
       </c>
-      <c r="E89">
+      <c r="E91">
         <v>355610.364944759</v>
       </c>
-      <c r="F89">
+      <c r="F91">
         <v>0.75267772890587503</v>
       </c>
-      <c r="G89">
+      <c r="G91">
         <v>25765.651662743599</v>
       </c>
-      <c r="H89">
+      <c r="H91">
         <v>7150.9042815892099</v>
       </c>
-      <c r="I89">
+      <c r="I91">
         <v>5144.3184852884797</v>
       </c>
-      <c r="J89">
+      <c r="J91">
         <v>38060.874429621297</v>
       </c>
-      <c r="K89">
+      <c r="K91">
         <v>64168.339029134899</v>
       </c>
-      <c r="L89">
+      <c r="L91">
         <v>19539.954214541001</v>
       </c>
-      <c r="M89">
+      <c r="M91">
         <v>24338.851661831999</v>
       </c>
-      <c r="N89">
+      <c r="N91">
         <v>1010.46273302954</v>
       </c>
-      <c r="O89">
-        <v>0</v>
-      </c>
-      <c r="P89">
-        <f t="shared" si="19"/>
+      <c r="O91">
+        <v>0</v>
+      </c>
+      <c r="P91">
+        <f t="shared" si="20"/>
         <v>267678.15388715523</v>
       </c>
-      <c r="Q89">
+      <c r="Q91">
         <v>1597.68911089628</v>
       </c>
-      <c r="R89">
+      <c r="R91">
         <v>13084.0423994256</v>
       </c>
-      <c r="S89">
+      <c r="S91">
         <v>467.28722855091399</v>
       </c>
-      <c r="T89">
+      <c r="T91">
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A90" t="s">
+    <row r="92" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A92" t="s">
         <v>22</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B92" t="s">
         <v>35</v>
       </c>
-      <c r="C90" t="s">
+      <c r="C92" t="s">
         <v>35</v>
       </c>
-      <c r="D90" t="s">
+      <c r="D92" t="s">
         <v>36</v>
       </c>
-      <c r="E90" t="s">
+      <c r="E92" t="s">
         <v>36</v>
       </c>
-      <c r="F90" t="s">
+      <c r="F92" t="s">
         <v>36</v>
       </c>
-      <c r="G90" s="4">
+      <c r="G92" s="4">
         <v>28838</v>
       </c>
-      <c r="H90">
+      <c r="H92">
         <v>7567.5</v>
       </c>
-      <c r="I90">
+      <c r="I92">
         <v>13764.1</v>
       </c>
-      <c r="J90">
+      <c r="J92">
         <v>50169.7</v>
       </c>
-      <c r="K90" t="s">
+      <c r="K92" t="s">
         <v>64</v>
       </c>
-      <c r="L90" t="s">
+      <c r="L92" t="s">
         <v>64</v>
       </c>
-      <c r="M90" t="s">
+      <c r="M92" t="s">
         <v>64</v>
       </c>
-      <c r="N90" t="s">
+      <c r="N92" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.4"/>
-    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A92" s="1" t="s">
+    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.4"/>
+    <row r="94" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A94" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G92" s="4"/>
-      <c r="P92" t="s">
+      <c r="G94" s="4"/>
+      <c r="P94" t="s">
         <v>15</v>
       </c>
-      <c r="Q92" t="s">
+      <c r="Q94" t="s">
         <v>16</v>
       </c>
-      <c r="R92" t="s">
+      <c r="R94" t="s">
         <v>17</v>
       </c>
-      <c r="S92" t="s">
+      <c r="S94" t="s">
         <v>18</v>
       </c>
-      <c r="T92" t="s">
+      <c r="T94" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A93" t="s">
-        <v>0</v>
-      </c>
-      <c r="B93" t="s">
+    <row r="95" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A95" t="s">
+        <v>0</v>
+      </c>
+      <c r="B95" t="s">
         <v>1</v>
       </c>
-      <c r="C93" t="s">
+      <c r="C95" t="s">
         <v>2</v>
       </c>
-      <c r="D93" t="s">
+      <c r="D95" t="s">
         <v>3</v>
       </c>
-      <c r="E93" t="s">
+      <c r="E95" t="s">
         <v>4</v>
       </c>
-      <c r="F93" t="s">
+      <c r="F95" t="s">
         <v>5</v>
       </c>
-      <c r="G93" s="4" t="s">
+      <c r="G95" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H93" t="s">
+      <c r="H95" t="s">
         <v>7</v>
       </c>
-      <c r="I93" t="s">
+      <c r="I95" t="s">
         <v>8</v>
       </c>
-      <c r="J93" t="s">
+      <c r="J95" t="s">
         <v>9</v>
       </c>
-      <c r="K93" t="s">
+      <c r="K95" t="s">
         <v>10</v>
       </c>
-      <c r="L93" t="s">
+      <c r="L95" t="s">
         <v>11</v>
       </c>
-      <c r="M93" t="s">
+      <c r="M95" t="s">
         <v>12</v>
       </c>
-      <c r="N93" t="s">
+      <c r="N95" t="s">
         <v>13</v>
       </c>
-      <c r="O93" t="s">
+      <c r="O95" t="s">
         <v>14</v>
       </c>
-      <c r="P93">
+      <c r="P95">
         <v>63734.6679</v>
       </c>
-      <c r="Q93">
+      <c r="Q95">
         <v>1078.4492829999999</v>
       </c>
-      <c r="R93">
+      <c r="R95">
         <v>624.70352849999995</v>
       </c>
-      <c r="S93">
+      <c r="S95">
         <v>13.014656840000001</v>
       </c>
-      <c r="T93">
+      <c r="T95">
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="G94" s="4"/>
-    </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A95" t="s">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="G96" s="4"/>
+    </row>
+    <row r="97" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A97" t="s">
         <v>20</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B97" t="s">
         <v>21</v>
       </c>
-      <c r="C95">
+      <c r="C97">
         <v>4</v>
       </c>
-      <c r="D95">
-        <f>J95+K95+L95+M95+N95</f>
+      <c r="D97">
+        <f>J97+K97+L97+M97+N97</f>
         <v>121563.11893886774</v>
       </c>
-      <c r="E95">
+      <c r="E97">
         <v>306531.77686027403</v>
       </c>
-      <c r="F95">
+      <c r="F97">
         <v>0.78839751879627895</v>
       </c>
-      <c r="G95">
+      <c r="G97">
         <v>19075.241421310599</v>
       </c>
-      <c r="H95">
+      <c r="H97">
         <v>6261.96818995999</v>
       </c>
-      <c r="I95">
+      <c r="I97">
         <v>1707.4548259942601</v>
       </c>
-      <c r="J95">
+      <c r="J97">
         <v>27044.664437264801</v>
       </c>
-      <c r="K95">
+      <c r="K97">
         <v>55296.129476701703</v>
       </c>
-      <c r="L95">
+      <c r="L97">
         <v>16799.683918922601</v>
       </c>
-      <c r="M95">
+      <c r="M97">
         <v>20976.431949083999</v>
       </c>
-      <c r="N95">
+      <c r="N97">
         <v>1446.20915689464</v>
       </c>
-      <c r="O95">
-        <v>0</v>
-      </c>
-      <c r="P95">
-        <f t="shared" ref="P95" si="20">D95+$P$1</f>
+      <c r="O97">
+        <v>0</v>
+      </c>
+      <c r="P97">
+        <f t="shared" ref="P97" si="21">D97+$P$1</f>
         <v>242122.79075786425</v>
       </c>
-      <c r="Q95">
+      <c r="Q97">
         <v>1421.8975872168901</v>
       </c>
-      <c r="R95">
+      <c r="R97">
         <v>16926.965777071098</v>
       </c>
-      <c r="S95">
+      <c r="S97">
         <v>248.92596730986901</v>
       </c>
-      <c r="T95">
+      <c r="T97">
         <v>-0.61547468554465901</v>
       </c>
-      <c r="U95">
+      <c r="U97">
         <v>31937.310450388199</v>
       </c>
-      <c r="V95">
+      <c r="V97">
         <v>319.37310450388202</v>
       </c>
     </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A96" s="3" t="s">
+    <row r="98" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A98" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B98" t="s">
         <v>35</v>
       </c>
-      <c r="C96" t="s">
+      <c r="C98" t="s">
         <v>35</v>
       </c>
-      <c r="D96" t="s">
+      <c r="D98" t="s">
         <v>36</v>
       </c>
-      <c r="E96" t="s">
+      <c r="E98" t="s">
         <v>36</v>
       </c>
-      <c r="F96" t="s">
+      <c r="F98" t="s">
         <v>36</v>
       </c>
-      <c r="G96" s="10">
+      <c r="G98" s="10">
         <v>21558</v>
       </c>
-      <c r="H96">
+      <c r="H98">
         <v>7337</v>
       </c>
-      <c r="I96">
+      <c r="I98">
         <v>3883</v>
       </c>
-      <c r="J96" s="10">
-        <f>G96+H96+I96</f>
+      <c r="J98" s="10">
+        <f>G98+H98+I98</f>
         <v>32778</v>
       </c>
-      <c r="K96" t="s">
+      <c r="K98" t="s">
         <v>64</v>
       </c>
-      <c r="L96" t="s">
+      <c r="L98" t="s">
         <v>64</v>
       </c>
-      <c r="M96" t="s">
+      <c r="M98" t="s">
         <v>64</v>
       </c>
-      <c r="N96" t="s">
+      <c r="N98" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="97" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A97" s="2"/>
-      <c r="G97" s="4"/>
-    </row>
     <row r="99" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A99" s="1" t="s">
+      <c r="A99" s="2"/>
+      <c r="G99" s="4"/>
+    </row>
+    <row r="101" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A101" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A100" t="s">
+    <row r="102" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A102" t="s">
         <v>22</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B102" t="s">
         <v>23</v>
       </c>
-      <c r="C100">
-        <v>0</v>
-      </c>
-      <c r="D100">
-        <f>J100+K100+L100+M100+N100</f>
+      <c r="C102">
+        <v>0</v>
+      </c>
+      <c r="D102">
+        <f>J102+K102+L102+M102+N102</f>
         <v>144641.57326653044</v>
       </c>
-      <c r="E100">
+      <c r="E102">
         <v>282179.67123287602</v>
       </c>
-      <c r="F100">
+      <c r="F102">
         <v>0.85636894399557495</v>
       </c>
-      <c r="G100">
+      <c r="G102">
         <v>20627.43117349</v>
       </c>
-      <c r="H100">
+      <c r="H102">
         <v>4930.8542128783001</v>
       </c>
-      <c r="I100">
+      <c r="I102">
         <v>9095.1262763121395</v>
       </c>
-      <c r="J100">
+      <c r="J102">
         <v>34653.411662680403</v>
       </c>
-      <c r="K100">
+      <c r="K102">
         <v>50843.184005923598</v>
       </c>
-      <c r="L100">
+      <c r="L102">
         <f>L4*(1.08/0.43)</f>
         <v>38437.447108478234</v>
       </c>
-      <c r="M100">
+      <c r="M102">
         <v>19297.5304894482</v>
       </c>
-      <c r="N100">
+      <c r="N102">
         <v>1410</v>
       </c>
-      <c r="O100">
-        <v>0</v>
-      </c>
-      <c r="P100">
-        <f t="shared" ref="P100" si="21">D100+$P$1</f>
+      <c r="O102">
+        <v>0</v>
+      </c>
+      <c r="P102">
+        <f t="shared" ref="P102" si="22">D102+$P$1</f>
         <v>265201.24508552696</v>
-      </c>
-    </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A101" t="s">
-        <v>22</v>
-      </c>
-      <c r="B101" t="s">
-        <v>21</v>
-      </c>
-      <c r="C101">
-        <v>4</v>
-      </c>
-      <c r="D101">
-        <f>J101+K101+L101+M101+N101</f>
-        <v>141686.61445013408</v>
-      </c>
-      <c r="E101">
-        <v>282179.70347192901</v>
-      </c>
-      <c r="F101">
-        <v>0.92782505226740197</v>
-      </c>
-      <c r="G101">
-        <v>19831.065688191899</v>
-      </c>
-      <c r="H101">
-        <v>6230.6791730567802</v>
-      </c>
-      <c r="I101">
-        <v>4871.4166947967997</v>
-      </c>
-      <c r="J101">
-        <v>30933.161556045401</v>
-      </c>
-      <c r="K101">
-        <v>50937.4505788346</v>
-      </c>
-      <c r="L101">
-        <v>39073.7116581429</v>
-      </c>
-      <c r="M101">
-        <v>19317.091802737999</v>
-      </c>
-      <c r="N101">
-        <v>1425.19885437316</v>
-      </c>
-      <c r="O101">
-        <v>0</v>
-      </c>
-      <c r="P101">
-        <f t="shared" ref="P101" si="22">D101+$P$1</f>
-        <v>262246.28626913059</v>
-      </c>
-      <c r="Q101">
-        <v>1392.0880151674601</v>
-      </c>
-      <c r="R101">
-        <v>14195.8581733913</v>
-      </c>
-      <c r="S101">
-        <v>112.66554105866101</v>
-      </c>
-      <c r="T101">
-        <v>-1.52076853589591</v>
-      </c>
-      <c r="U101">
-        <v>12183.2216733653</v>
-      </c>
-      <c r="V101">
-        <v>290.07670650869801</v>
-      </c>
-    </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="K102">
-        <f>SUM(K100:M100)-SUM(K101:M101)</f>
-        <v>-750.09243586547382</v>
       </c>
     </row>
     <row r="103" spans="1:22" x14ac:dyDescent="0.4">
@@ -5965,423 +5988,413 @@
         <v>22</v>
       </c>
       <c r="B103" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C103">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D103">
         <f>J103+K103+L103+M103+N103</f>
+        <v>141686.61445013408</v>
+      </c>
+      <c r="E103">
+        <v>282179.70347192901</v>
+      </c>
+      <c r="F103">
+        <v>0.92782505226740197</v>
+      </c>
+      <c r="G103">
+        <v>19831.065688191899</v>
+      </c>
+      <c r="H103">
+        <v>6230.6791730567802</v>
+      </c>
+      <c r="I103">
+        <v>4871.4166947967997</v>
+      </c>
+      <c r="J103">
+        <v>30933.161556045401</v>
+      </c>
+      <c r="K103">
+        <v>50937.4505788346</v>
+      </c>
+      <c r="L103">
+        <v>39073.7116581429</v>
+      </c>
+      <c r="M103">
+        <v>19317.091802737999</v>
+      </c>
+      <c r="N103">
+        <v>1425.19885437316</v>
+      </c>
+      <c r="O103">
+        <v>0</v>
+      </c>
+      <c r="P103">
+        <f t="shared" ref="P103" si="23">D103+$P$1</f>
+        <v>262246.28626913059</v>
+      </c>
+      <c r="Q103">
+        <v>1392.0880151674601</v>
+      </c>
+      <c r="R103">
+        <v>14195.8581733913</v>
+      </c>
+      <c r="S103">
+        <v>112.66554105866101</v>
+      </c>
+      <c r="T103">
+        <v>-1.52076853589591</v>
+      </c>
+      <c r="U103">
+        <v>12183.2216733653</v>
+      </c>
+      <c r="V103">
+        <v>290.07670650869801</v>
+      </c>
+    </row>
+    <row r="104" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="K104">
+        <f>SUM(K102:M102)-SUM(K103:M103)</f>
+        <v>-750.09243586547382</v>
+      </c>
+    </row>
+    <row r="105" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A105" t="s">
+        <v>22</v>
+      </c>
+      <c r="B105" t="s">
+        <v>23</v>
+      </c>
+      <c r="C105">
+        <v>0</v>
+      </c>
+      <c r="D105">
+        <f>J105+K105+L105+M105+N105</f>
         <v>182723.11808696718</v>
       </c>
-      <c r="E103">
+      <c r="E105">
         <v>282179.67123287602</v>
       </c>
-      <c r="F103">
+      <c r="F105">
         <v>0.85636894399557495</v>
       </c>
-      <c r="G103">
+      <c r="G105">
         <v>20627.43117349</v>
       </c>
-      <c r="H103">
+      <c r="H105">
         <v>4930.8542128783001</v>
       </c>
-      <c r="I103">
+      <c r="I105">
         <v>9095.1262763121395</v>
       </c>
-      <c r="J103">
+      <c r="J105">
         <v>34653.411662680403</v>
       </c>
-      <c r="K103">
+      <c r="K105">
         <v>50843.184005923598</v>
       </c>
-      <c r="L103">
+      <c r="L105">
         <f>L4*(2.15/0.43)</f>
         <v>76518.991928914998</v>
       </c>
-      <c r="M103">
+      <c r="M105">
         <v>19297.5304894482</v>
       </c>
-      <c r="N103">
+      <c r="N105">
         <v>1410</v>
       </c>
-      <c r="P103">
-        <f t="shared" ref="P103:P104" si="23">D103+$P$1</f>
+      <c r="P105">
+        <f t="shared" ref="P105:P106" si="24">D105+$P$1</f>
         <v>303282.7899059637</v>
       </c>
     </row>
-    <row r="104" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A104" t="s">
+    <row r="106" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A106" t="s">
         <v>22</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B106" t="s">
         <v>21</v>
       </c>
-      <c r="C104">
+      <c r="C106">
         <v>4</v>
       </c>
-      <c r="D104" s="13">
-        <f>J104+K104+L104+M104+N104</f>
+      <c r="D106" s="13">
+        <f>J106+K106+L106+M106+N106</f>
         <v>180164.72653261331</v>
       </c>
-      <c r="E104" s="13">
+      <c r="E106" s="13">
         <v>282179.67123285698</v>
       </c>
-      <c r="F104" s="12">
+      <c r="F106" s="12">
         <v>1.0641670739695701</v>
       </c>
-      <c r="G104" s="13">
+      <c r="G106" s="13">
         <v>19863.1783561796</v>
       </c>
-      <c r="H104" s="13">
+      <c r="H106" s="13">
         <v>6506.5697069746102</v>
       </c>
-      <c r="I104" s="13">
+      <c r="I106" s="13">
         <v>4873.61028676154</v>
       </c>
-      <c r="J104" s="13">
+      <c r="J106" s="13">
         <v>31243.358349915699</v>
       </c>
-      <c r="K104" s="13">
+      <c r="K106" s="13">
         <v>50899.9452054371</v>
       </c>
-      <c r="L104" s="13">
+      <c r="L106" s="13">
         <v>77281.720548983998</v>
       </c>
-      <c r="M104" s="13">
+      <c r="M106" s="13">
         <v>19309.308438346699</v>
       </c>
-      <c r="N104" s="13">
+      <c r="N106" s="13">
         <v>1430.39398992981</v>
       </c>
-      <c r="O104">
-        <v>0</v>
-      </c>
-      <c r="P104">
-        <f t="shared" si="23"/>
+      <c r="O106">
+        <v>0</v>
+      </c>
+      <c r="P106">
+        <f t="shared" si="24"/>
         <v>300724.39835160982</v>
       </c>
-      <c r="Q104" s="4">
+      <c r="Q106" s="4">
         <v>1453.7288077599201</v>
       </c>
-      <c r="R104">
+      <c r="R106">
         <v>14136.371585592</v>
       </c>
-      <c r="S104" s="4">
+      <c r="S106" s="4">
         <v>107.91123347780101</v>
       </c>
-      <c r="T104" s="12">
+      <c r="T106" s="12">
         <v>-4.2490908058638102</v>
       </c>
-      <c r="U104">
+      <c r="U106">
         <v>13013.5923280234</v>
       </c>
-      <c r="V104" s="4">
+      <c r="V106" s="4">
         <v>351.71871156820202</v>
       </c>
     </row>
-    <row r="105" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="K105" s="13">
-        <f>SUM(K103:M103)-SUM(K104:M104)</f>
+    <row r="107" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="K107" s="13">
+        <f>SUM(K105:M105)-SUM(K106:M106)</f>
         <v>-831.26776848098962</v>
       </c>
     </row>
-    <row r="106" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A106" s="1" t="s">
+    <row r="108" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A108" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="K106" s="13"/>
-    </row>
-    <row r="107" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A107" t="s">
+      <c r="K108" s="13"/>
+    </row>
+    <row r="109" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A109" t="s">
         <v>22</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B109" t="s">
         <v>23</v>
       </c>
-      <c r="C107">
+      <c r="C109">
         <v>4</v>
       </c>
-      <c r="D107" s="13">
-        <f>J107+K107+L107+M107+N107</f>
+      <c r="D109" s="13">
+        <f>J109+K109+L109+M109+N109</f>
         <v>119726.39965297376</v>
       </c>
-      <c r="E107">
+      <c r="E109">
         <v>282179.83224964398</v>
       </c>
-      <c r="F107">
+      <c r="F109">
         <v>0.84996419881982699</v>
       </c>
-      <c r="G107">
+      <c r="G109">
         <v>20303.288104589901</v>
       </c>
-      <c r="H107">
+      <c r="H109">
         <v>6543.2205338351096</v>
       </c>
-      <c r="I107">
+      <c r="I109">
         <v>5999.24631325068</v>
       </c>
-      <c r="J107">
+      <c r="J109">
         <v>32845.754951675699</v>
       </c>
-      <c r="K107">
+      <c r="K109">
         <v>50843.330071946802</v>
       </c>
-      <c r="L107">
+      <c r="L109">
         <v>15304.121701009901</v>
       </c>
-      <c r="M107">
+      <c r="M109">
         <v>19297.5657896679</v>
       </c>
-      <c r="N107">
+      <c r="N109">
         <v>1435.62713867346</v>
       </c>
-      <c r="O107">
-        <v>0</v>
-      </c>
-      <c r="P107">
-        <f t="shared" ref="P107:P108" si="24">D107+$P$1</f>
+      <c r="O109">
+        <v>0</v>
+      </c>
+      <c r="P109">
+        <f t="shared" ref="P109:P110" si="25">D109+$P$1</f>
         <v>240286.0714719703</v>
       </c>
-      <c r="Q107">
+      <c r="Q109">
         <v>1461.9175121692599</v>
       </c>
-      <c r="R107">
+      <c r="R109">
         <v>30796.244401685999</v>
       </c>
-      <c r="S107">
+      <c r="S109">
         <v>375.56395611812201</v>
       </c>
-      <c r="T107">
+      <c r="T109">
         <v>1.20664176507714E-2</v>
       </c>
-      <c r="U107">
+      <c r="U109">
         <v>30890.848067330899</v>
       </c>
-      <c r="V107">
+      <c r="V109">
         <v>359.195907759661</v>
       </c>
     </row>
-    <row r="108" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A108" t="s">
+    <row r="110" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A110" t="s">
         <v>22</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B110" t="s">
         <v>21</v>
       </c>
-      <c r="C108">
+      <c r="C110">
         <v>4</v>
       </c>
-      <c r="D108" s="13">
-        <f>J108+K108+L108+M108+N108</f>
+      <c r="D110" s="13">
+        <f>J110+K110+L110+M110+N110</f>
         <v>118661.22865756074</v>
       </c>
-      <c r="E108">
+      <c r="E110">
         <v>282195.464864693</v>
       </c>
-      <c r="F108">
+      <c r="F110">
         <v>0.84615181718922305</v>
       </c>
-      <c r="G108">
+      <c r="G110">
         <v>20110.907995096401</v>
       </c>
-      <c r="H108">
+      <c r="H110">
         <v>6540.2066794450602</v>
       </c>
-      <c r="I108">
+      <c r="I110">
         <v>4890.2435679090904</v>
       </c>
-      <c r="J108">
+      <c r="J110">
         <v>31541.358242450598</v>
       </c>
-      <c r="K108">
+      <c r="K110">
         <v>50907.023134659299</v>
       </c>
-      <c r="L108">
+      <c r="L110">
         <v>15468.5747825788</v>
       </c>
-      <c r="M108">
+      <c r="M110">
         <v>19311.266711247299</v>
       </c>
-      <c r="N108">
+      <c r="N110">
         <v>1433.00578662475</v>
       </c>
-      <c r="O108">
-        <v>0</v>
-      </c>
-      <c r="P108">
-        <f t="shared" si="24"/>
+      <c r="O110">
+        <v>0</v>
+      </c>
+      <c r="P110">
+        <f t="shared" si="25"/>
         <v>239220.90047655726</v>
       </c>
-      <c r="Q108">
+      <c r="Q110">
         <v>1461.2441424594499</v>
       </c>
-      <c r="R108">
+      <c r="R110">
         <v>30869.812631599802</v>
       </c>
-      <c r="S108">
+      <c r="S110">
         <v>411.59750175466399</v>
       </c>
-      <c r="T108">
+      <c r="T110">
         <v>4.6542923975130698E-2</v>
       </c>
-      <c r="U108">
+      <c r="U110">
         <v>30784.7301446001</v>
       </c>
-      <c r="V108">
+      <c r="V110">
         <v>331.01860370537798</v>
       </c>
     </row>
-    <row r="109" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="D109" s="13">
-        <f>D108-D31</f>
+    <row r="111" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="D111" s="13">
+        <f>D110-D31</f>
         <v>870.81314264753019</v>
       </c>
-      <c r="E109" s="13">
-        <f t="shared" ref="E109:N109" si="25">E108-E31</f>
+      <c r="E111" s="13">
+        <f t="shared" ref="E111:N111" si="26">E110-E31</f>
         <v>15.79363181698136</v>
       </c>
-      <c r="F109" s="13">
-        <f t="shared" si="25"/>
+      <c r="F111" s="13">
+        <f t="shared" si="26"/>
         <v>3.0492754563130609E-3</v>
       </c>
-      <c r="G109" s="13">
-        <f t="shared" si="25"/>
+      <c r="G111" s="13">
+        <f t="shared" si="26"/>
         <v>270.37094434599931</v>
       </c>
-      <c r="H109" s="13">
-        <f t="shared" si="25"/>
+      <c r="H111" s="13">
+        <f t="shared" si="26"/>
         <v>1259.5735968278204</v>
       </c>
-      <c r="I109" s="13">
-        <f t="shared" si="25"/>
+      <c r="I111" s="13">
+        <f t="shared" si="26"/>
         <v>12.753618583180469</v>
       </c>
-      <c r="J109" s="13">
-        <f t="shared" si="25"/>
+      <c r="J111" s="13">
+        <f t="shared" si="26"/>
         <v>1542.6981597569975</v>
       </c>
-      <c r="K109" s="13">
-        <f t="shared" si="25"/>
+      <c r="K111" s="13">
+        <f t="shared" si="26"/>
         <v>-170.1127457354014</v>
       </c>
-      <c r="L109" s="13">
-        <f t="shared" si="25"/>
+      <c r="L111" s="13">
+        <f t="shared" si="26"/>
         <v>-463.96926584500034</v>
       </c>
-      <c r="M109" s="13">
-        <f t="shared" si="25"/>
+      <c r="M111" s="13">
+        <f t="shared" si="26"/>
         <v>-34.808792153802642</v>
       </c>
-      <c r="N109" s="13">
-        <f t="shared" si="25"/>
+      <c r="N111" s="13">
+        <f t="shared" si="26"/>
         <v>-2.9942133752499558</v>
       </c>
     </row>
-    <row r="110" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="D110" s="13"/>
-      <c r="E110" s="13"/>
-      <c r="F110" s="13"/>
-      <c r="G110" s="13"/>
-      <c r="H110" s="13"/>
-      <c r="I110" s="13"/>
-      <c r="J110" s="13"/>
-      <c r="K110" s="13"/>
-      <c r="L110" s="13"/>
-      <c r="M110" s="13"/>
-      <c r="N110" s="13"/>
-    </row>
-    <row r="111" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A111" s="1" t="s">
+    <row r="112" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="D112" s="13"/>
+      <c r="E112" s="13"/>
+      <c r="F112" s="13"/>
+      <c r="G112" s="13"/>
+      <c r="H112" s="13"/>
+      <c r="I112" s="13"/>
+      <c r="J112" s="13"/>
+      <c r="K112" s="13"/>
+      <c r="L112" s="13"/>
+      <c r="M112" s="13"/>
+      <c r="N112" s="13"/>
+    </row>
+    <row r="113" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A113" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D111" s="13"/>
-      <c r="E111" s="13"/>
-      <c r="F111" s="13"/>
-      <c r="G111" s="13"/>
-      <c r="H111" s="13"/>
-      <c r="I111" s="13"/>
-      <c r="J111" s="13"/>
-      <c r="K111" s="13"/>
-      <c r="L111" s="13"/>
-      <c r="M111" s="13"/>
-      <c r="N111" s="13"/>
-    </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A112" t="s">
-        <v>22</v>
-      </c>
-      <c r="B112" t="s">
-        <v>21</v>
-      </c>
-      <c r="C112">
-        <v>4</v>
-      </c>
-      <c r="D112" s="13">
-        <f>J112+K112+L112+M112+N112</f>
-        <v>113976.01616633293</v>
-      </c>
-      <c r="E112">
-        <v>282179.67123285797</v>
-      </c>
-      <c r="F112">
-        <v>0.82949143613233001</v>
-      </c>
-      <c r="G112">
-        <v>19739.4095985942</v>
-      </c>
-      <c r="H112">
-        <v>6280.2265894411403</v>
-      </c>
-      <c r="I112">
-        <v>0</v>
-      </c>
-      <c r="J112">
-        <v>26019.6361880353</v>
-      </c>
-      <c r="K112">
-        <v>50944.945205466604</v>
-      </c>
-      <c r="L112">
-        <v>15577.281609678699</v>
-      </c>
-      <c r="M112">
-        <v>19971.775208230301</v>
-      </c>
-      <c r="N112">
-        <v>1462.3779549220301</v>
-      </c>
-      <c r="O112">
-        <v>0</v>
-      </c>
-      <c r="P112">
-        <f t="shared" ref="P112" si="26">D112+$P$1</f>
-        <v>234535.68798532945</v>
-      </c>
-      <c r="Q112">
-        <v>1403.15815187257</v>
-      </c>
-      <c r="R112">
-        <v>34638.685534293101</v>
-      </c>
-      <c r="S112">
-        <v>865.96713835732805</v>
-      </c>
-      <c r="T112">
-        <v>0.1767383415172</v>
-      </c>
-      <c r="U112">
-        <v>38493.267558113897</v>
-      </c>
-      <c r="V112">
-        <v>300.72865279776499</v>
-      </c>
-    </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="D113" s="12">
-        <f>(D112-D4)</f>
-        <v>-7531.9083775022591</v>
-      </c>
+      <c r="D113" s="13"/>
       <c r="E113" s="13"/>
       <c r="F113" s="13"/>
       <c r="G113" s="13"/>
@@ -6393,489 +6406,576 @@
       <c r="M113" s="13"/>
       <c r="N113" s="13"/>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="D114" s="13"/>
-      <c r="E114" s="13"/>
-      <c r="F114" s="13"/>
-      <c r="G114" s="13"/>
-      <c r="H114" s="13"/>
-      <c r="I114" s="13"/>
-      <c r="J114" s="13"/>
-      <c r="K114" s="13"/>
-      <c r="L114" s="13"/>
-      <c r="M114" s="13"/>
-      <c r="N114" s="13"/>
-    </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A115" s="7" t="s">
+    <row r="114" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A114" t="s">
+        <v>22</v>
+      </c>
+      <c r="B114" t="s">
+        <v>21</v>
+      </c>
+      <c r="C114">
+        <v>4</v>
+      </c>
+      <c r="D114" s="13">
+        <f>J114+K114+L114+M114+N114</f>
+        <v>113976.01616633293</v>
+      </c>
+      <c r="E114">
+        <v>282179.67123285797</v>
+      </c>
+      <c r="F114">
+        <v>0.82949143613233001</v>
+      </c>
+      <c r="G114">
+        <v>19739.4095985942</v>
+      </c>
+      <c r="H114">
+        <v>6280.2265894411403</v>
+      </c>
+      <c r="I114">
+        <v>0</v>
+      </c>
+      <c r="J114">
+        <v>26019.6361880353</v>
+      </c>
+      <c r="K114">
+        <v>50944.945205466604</v>
+      </c>
+      <c r="L114">
+        <v>15577.281609678699</v>
+      </c>
+      <c r="M114">
+        <v>19971.775208230301</v>
+      </c>
+      <c r="N114">
+        <v>1462.3779549220301</v>
+      </c>
+      <c r="O114">
+        <v>0</v>
+      </c>
+      <c r="P114">
+        <f t="shared" ref="P114" si="27">D114+$P$1</f>
+        <v>234535.68798532945</v>
+      </c>
+      <c r="Q114">
+        <v>1403.15815187257</v>
+      </c>
+      <c r="R114">
+        <v>34638.685534293101</v>
+      </c>
+      <c r="S114">
+        <v>865.96713835732805</v>
+      </c>
+      <c r="T114">
+        <v>0.1767383415172</v>
+      </c>
+      <c r="U114">
+        <v>38493.267558113897</v>
+      </c>
+      <c r="V114">
+        <v>300.72865279776499</v>
+      </c>
+    </row>
+    <row r="115" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="D115" s="12">
+        <f>(D114-D4)</f>
+        <v>-7531.9083775022591</v>
+      </c>
+      <c r="E115" s="13"/>
+      <c r="F115" s="13"/>
+      <c r="G115" s="13"/>
+      <c r="H115" s="13"/>
+      <c r="I115" s="13"/>
+      <c r="J115" s="13"/>
+      <c r="K115" s="13"/>
+      <c r="L115" s="13"/>
+      <c r="M115" s="13"/>
+      <c r="N115" s="13"/>
+    </row>
+    <row r="116" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="D116" s="13"/>
+      <c r="E116" s="13"/>
+      <c r="F116" s="13"/>
+      <c r="G116" s="13"/>
+      <c r="H116" s="13"/>
+      <c r="I116" s="13"/>
+      <c r="J116" s="13"/>
+      <c r="K116" s="13"/>
+      <c r="L116" s="13"/>
+      <c r="M116" s="13"/>
+      <c r="N116" s="13"/>
+    </row>
+    <row r="117" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A117" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A116" t="s">
+    <row r="118" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A118" t="s">
         <v>32</v>
       </c>
-      <c r="B116" t="s">
+      <c r="B118" t="s">
         <v>33</v>
       </c>
-      <c r="C116" t="s">
+      <c r="C118" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A117">
-        <v>20</v>
-      </c>
-      <c r="B117">
-        <v>60</v>
-      </c>
-      <c r="C117">
-        <v>2</v>
-      </c>
-      <c r="D117">
-        <f t="shared" ref="D117:D123" si="27">J117+K117+L117+M117+N117</f>
-        <v>120712.69088313227</v>
-      </c>
-      <c r="E117">
-        <v>282179.67123285501</v>
-      </c>
-      <c r="F117">
-        <v>0.854946898908852</v>
-      </c>
-      <c r="G117">
-        <v>18681.222424938602</v>
-      </c>
-      <c r="H117">
-        <v>5354.6114985546601</v>
-      </c>
-      <c r="I117">
-        <v>8156.08309050551</v>
-      </c>
-      <c r="J117">
-        <v>32191.917013998798</v>
-      </c>
-      <c r="K117">
-        <v>51372.124296964801</v>
-      </c>
-      <c r="L117">
-        <v>16725.325417965501</v>
-      </c>
-      <c r="M117">
-        <v>19407.285599838699</v>
-      </c>
-      <c r="N117">
-        <v>1016.03855436447</v>
-      </c>
-      <c r="O117">
-        <v>0</v>
-      </c>
-      <c r="P117">
-        <f t="shared" ref="P117:P123" si="28">D117+$P$1</f>
-        <v>241272.36270212877</v>
-      </c>
-      <c r="Q117">
-        <v>1192.7637589594799</v>
-      </c>
-      <c r="R117">
-        <v>19736.206339365101</v>
-      </c>
-      <c r="S117">
-        <v>481.37088632597801</v>
-      </c>
-      <c r="T117" s="6">
-        <v>0.12591688076390301</v>
-      </c>
-    </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A118">
-        <v>20</v>
-      </c>
-      <c r="B118">
-        <v>50</v>
-      </c>
-      <c r="C118">
-        <v>2</v>
-      </c>
-      <c r="D118">
-        <f t="shared" si="27"/>
-        <v>119392.42354269064</v>
-      </c>
-      <c r="E118">
-        <v>282254.81855225202</v>
-      </c>
-      <c r="F118">
-        <v>0.85006146065890897</v>
-      </c>
-      <c r="G118">
-        <v>19407.840072768398</v>
-      </c>
-      <c r="H118">
-        <v>5891.8301217549197</v>
-      </c>
-      <c r="I118">
-        <v>6659.4942697455399</v>
-      </c>
-      <c r="J118">
-        <v>31959.164464268899</v>
-      </c>
-      <c r="K118">
-        <v>51102.045942938203</v>
-      </c>
-      <c r="L118">
-        <v>15967.176494174801</v>
-      </c>
-      <c r="M118">
-        <v>19353.573908279199</v>
-      </c>
-      <c r="N118">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O118">
-        <v>0</v>
-      </c>
-      <c r="P118">
-        <f t="shared" si="28"/>
-        <v>239952.09536168716</v>
-      </c>
-      <c r="Q118">
-        <v>1312.43161993582</v>
-      </c>
-      <c r="R118">
-        <v>18377.616631847999</v>
-      </c>
-      <c r="S118">
-        <v>459.4404157962</v>
-      </c>
-      <c r="T118" s="6">
-        <v>0.14758705239613301</v>
-      </c>
-    </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="119" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A119">
         <v>20</v>
       </c>
       <c r="B119">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C119">
         <v>2</v>
       </c>
       <c r="D119">
-        <f t="shared" si="27"/>
-        <v>117777.02945340994</v>
+        <f t="shared" ref="D119:D125" si="28">J119+K119+L119+M119+N119</f>
+        <v>120712.69088313227</v>
       </c>
       <c r="E119">
-        <v>282179.67123287299</v>
+        <v>282179.67123285501</v>
       </c>
       <c r="F119">
-        <v>0.84456314023622803</v>
+        <v>0.854946898908852</v>
       </c>
       <c r="G119">
-        <v>19298.245593088301</v>
+        <v>18681.222424938602</v>
       </c>
       <c r="H119">
-        <v>5682.0016560700296</v>
+        <v>5354.6114985546601</v>
       </c>
       <c r="I119">
-        <v>5350.3346939491703</v>
+        <v>8156.08309050551</v>
       </c>
       <c r="J119">
-        <v>30330.5819431075</v>
+        <v>32191.917013998798</v>
       </c>
       <c r="K119">
-        <v>51097.733915068202</v>
+        <v>51372.124296964801</v>
       </c>
       <c r="L119">
-        <v>15987.901266609</v>
+        <v>16725.325417965501</v>
       </c>
       <c r="M119">
-        <v>19350.349595595701</v>
+        <v>19407.285599838699</v>
       </c>
       <c r="N119">
-        <v>1010.46273302954</v>
+        <v>1016.03855436447</v>
       </c>
       <c r="O119">
         <v>0</v>
       </c>
       <c r="P119">
-        <f t="shared" si="28"/>
-        <v>238336.70127240644</v>
+        <f t="shared" ref="P119:P125" si="29">D119+$P$1</f>
+        <v>241272.36270212877</v>
       </c>
       <c r="Q119">
-        <v>1265.6913868611</v>
+        <v>1192.7637589594799</v>
       </c>
       <c r="R119">
-        <v>17746.163883660702</v>
+        <v>19736.206339365101</v>
       </c>
       <c r="S119">
-        <v>507.03325381887902</v>
+        <v>481.37088632597801</v>
       </c>
       <c r="T119" s="6">
-        <v>-0.25983751983286502</v>
-      </c>
-    </row>
-    <row r="120" spans="1:20" x14ac:dyDescent="0.4">
+        <v>0.12591688076390301</v>
+      </c>
+    </row>
+    <row r="120" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A120">
         <v>20</v>
       </c>
       <c r="B120">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C120">
         <v>2</v>
       </c>
       <c r="D120">
-        <f t="shared" si="27"/>
-        <v>116625.1695160947</v>
+        <f t="shared" si="28"/>
+        <v>119392.42354269064</v>
       </c>
       <c r="E120">
-        <v>282182.50548365602</v>
+        <v>282254.81855225202</v>
       </c>
       <c r="F120">
-        <v>0.84045954058697003</v>
+        <v>0.85006146065890897</v>
       </c>
       <c r="G120">
-        <v>19302.752565837702</v>
+        <v>19407.840072768398</v>
       </c>
       <c r="H120">
-        <v>6226.5181629292701</v>
+        <v>5891.8301217549197</v>
       </c>
       <c r="I120">
-        <v>3974.5318253822402</v>
+        <v>6659.4942697455399</v>
       </c>
       <c r="J120">
-        <v>29503.802554149199</v>
+        <v>31959.164464268899</v>
       </c>
       <c r="K120">
-        <v>51013.610661725899</v>
+        <v>51102.045942938203</v>
       </c>
       <c r="L120">
-        <v>15760.601295416</v>
+        <v>15967.176494174801</v>
       </c>
       <c r="M120">
-        <v>19332.981882301501</v>
+        <v>19353.573908279199</v>
       </c>
       <c r="N120">
-        <v>1014.17312250211</v>
+        <v>1010.46273302954</v>
       </c>
       <c r="O120">
         <v>0</v>
       </c>
       <c r="P120">
+        <f t="shared" si="29"/>
+        <v>239952.09536168716</v>
+      </c>
+      <c r="Q120">
+        <v>1312.43161993582</v>
+      </c>
+      <c r="R120">
+        <v>18377.616631847999</v>
+      </c>
+      <c r="S120">
+        <v>459.4404157962</v>
+      </c>
+      <c r="T120" s="6">
+        <v>0.14758705239613301</v>
+      </c>
+    </row>
+    <row r="121" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A121">
+        <v>20</v>
+      </c>
+      <c r="B121">
+        <v>40</v>
+      </c>
+      <c r="C121">
+        <v>2</v>
+      </c>
+      <c r="D121">
         <f t="shared" si="28"/>
-        <v>237184.84133509122</v>
-      </c>
-      <c r="Q120">
-        <v>1386.9848841974899</v>
-      </c>
-      <c r="R120">
-        <v>18436.445202769701</v>
-      </c>
-      <c r="S120">
-        <v>209.50505912238299</v>
-      </c>
-      <c r="T120" s="6">
-        <v>0.28049716262959101</v>
-      </c>
-    </row>
-    <row r="121" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A121" s="3">
-        <v>20</v>
-      </c>
-      <c r="B121" s="3">
-        <v>20</v>
-      </c>
-      <c r="C121" s="3">
-        <v>2</v>
-      </c>
-      <c r="D121">
-        <f t="shared" si="27"/>
-        <v>115198.459983006</v>
+        <v>117777.02945340994</v>
       </c>
       <c r="E121">
-        <v>282179.67123297497</v>
+        <v>282179.67123287299</v>
       </c>
       <c r="F121">
-        <v>0.83541194997266699</v>
+        <v>0.84456314023622803</v>
       </c>
       <c r="G121">
-        <v>19351.2255529412</v>
+        <v>19298.245593088301</v>
       </c>
       <c r="H121">
-        <v>6002.0469674603501</v>
+        <v>5682.0016560700296</v>
       </c>
       <c r="I121">
-        <v>2645.4376652921501</v>
+        <v>5350.3346939491703</v>
       </c>
       <c r="J121">
-        <v>27998.710185693701</v>
+        <v>30330.5819431075</v>
       </c>
       <c r="K121">
-        <v>51033.4442867088</v>
+        <v>51097.733915068202</v>
       </c>
       <c r="L121">
-        <v>15815.1228903871</v>
+        <v>15987.901266609</v>
       </c>
       <c r="M121">
-        <v>19337.009497714302</v>
+        <v>19350.349595595701</v>
       </c>
       <c r="N121">
-        <v>1014.17312250211</v>
+        <v>1010.46273302954</v>
       </c>
       <c r="O121">
         <v>0</v>
       </c>
       <c r="P121">
-        <f t="shared" si="28"/>
-        <v>235758.13180200252</v>
+        <f t="shared" si="29"/>
+        <v>238336.70127240644</v>
       </c>
       <c r="Q121">
-        <v>1336.98290493166</v>
+        <v>1265.6913868611</v>
       </c>
       <c r="R121">
-        <v>18577.307877855899</v>
+        <v>17746.163883660702</v>
       </c>
       <c r="S121">
-        <v>432.030415764091</v>
+        <v>507.03325381887902</v>
       </c>
       <c r="T121" s="6">
-        <v>-0.122490141098651</v>
-      </c>
-    </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.4">
+        <v>-0.25983751983286502</v>
+      </c>
+    </row>
+    <row r="122" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A122">
         <v>20</v>
       </c>
       <c r="B122">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="C122">
         <v>2</v>
       </c>
       <c r="D122">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
+        <v>116625.1695160947</v>
+      </c>
+      <c r="E122">
+        <v>282182.50548365602</v>
+      </c>
+      <c r="F122">
+        <v>0.84045954058697003</v>
+      </c>
+      <c r="G122">
+        <v>19302.752565837702</v>
+      </c>
+      <c r="H122">
+        <v>6226.5181629292701</v>
+      </c>
+      <c r="I122">
+        <v>3974.5318253822402</v>
+      </c>
+      <c r="J122">
+        <v>29503.802554149199</v>
+      </c>
+      <c r="K122">
+        <v>51013.610661725899</v>
+      </c>
+      <c r="L122">
+        <v>15760.601295416</v>
+      </c>
+      <c r="M122">
+        <v>19332.981882301501</v>
+      </c>
+      <c r="N122">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O122">
+        <v>0</v>
+      </c>
+      <c r="P122">
+        <f t="shared" si="29"/>
+        <v>237184.84133509122</v>
+      </c>
+      <c r="Q122">
+        <v>1386.9848841974899</v>
+      </c>
+      <c r="R122">
+        <v>18436.445202769701</v>
+      </c>
+      <c r="S122">
+        <v>209.50505912238299</v>
+      </c>
+      <c r="T122" s="6">
+        <v>0.28049716262959101</v>
+      </c>
+    </row>
+    <row r="123" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A123" s="3">
+        <v>20</v>
+      </c>
+      <c r="B123" s="3">
+        <v>20</v>
+      </c>
+      <c r="C123" s="3">
+        <v>2</v>
+      </c>
+      <c r="D123">
+        <f t="shared" si="28"/>
+        <v>115198.459983006</v>
+      </c>
+      <c r="E123">
+        <v>282179.67123297497</v>
+      </c>
+      <c r="F123">
+        <v>0.83541194997266699</v>
+      </c>
+      <c r="G123">
+        <v>19351.2255529412</v>
+      </c>
+      <c r="H123">
+        <v>6002.0469674603501</v>
+      </c>
+      <c r="I123">
+        <v>2645.4376652921501</v>
+      </c>
+      <c r="J123">
+        <v>27998.710185693701</v>
+      </c>
+      <c r="K123">
+        <v>51033.4442867088</v>
+      </c>
+      <c r="L123">
+        <v>15815.1228903871</v>
+      </c>
+      <c r="M123">
+        <v>19337.009497714302</v>
+      </c>
+      <c r="N123">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O123">
+        <v>0</v>
+      </c>
+      <c r="P123">
+        <f t="shared" si="29"/>
+        <v>235758.13180200252</v>
+      </c>
+      <c r="Q123">
+        <v>1336.98290493166</v>
+      </c>
+      <c r="R123">
+        <v>18577.307877855899</v>
+      </c>
+      <c r="S123">
+        <v>432.030415764091</v>
+      </c>
+      <c r="T123" s="6">
+        <v>-0.122490141098651</v>
+      </c>
+    </row>
+    <row r="124" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A124">
+        <v>20</v>
+      </c>
+      <c r="B124">
+        <v>15</v>
+      </c>
+      <c r="C124">
+        <v>2</v>
+      </c>
+      <c r="D124">
+        <f t="shared" si="28"/>
         <v>114451.25872361983</v>
       </c>
-      <c r="E122">
+      <c r="E124">
         <v>282179.67123267101</v>
       </c>
-      <c r="F122">
+      <c r="F124">
         <v>0.83277713625127903</v>
       </c>
-      <c r="G122">
+      <c r="G124">
         <v>19390.977969205</v>
       </c>
-      <c r="H122">
+      <c r="H124">
         <v>5599.5405456203798</v>
       </c>
-      <c r="I122">
+      <c r="I124">
         <v>2128.1287863747102</v>
       </c>
-      <c r="J122">
+      <c r="J124">
         <v>27118.647301200101</v>
       </c>
-      <c r="K122">
+      <c r="K124">
         <v>51068.507704320902</v>
       </c>
-      <c r="L122">
+      <c r="L124">
         <v>15909.3558282099</v>
       </c>
-      <c r="M122">
+      <c r="M124">
         <v>19344.285156859401</v>
       </c>
-      <c r="N122">
+      <c r="N124">
         <v>1010.46273302954</v>
       </c>
-      <c r="O122">
-        <v>0</v>
-      </c>
-      <c r="P122">
+      <c r="O124">
+        <v>0</v>
+      </c>
+      <c r="P124">
+        <f t="shared" si="29"/>
+        <v>235010.93054261635</v>
+      </c>
+      <c r="Q124">
+        <v>1247.3228025527501</v>
+      </c>
+      <c r="R124">
+        <v>16417.502561416801</v>
+      </c>
+      <c r="S124">
+        <v>469.07150175476602</v>
+      </c>
+      <c r="T124" s="6">
+        <v>0.46004655114715598</v>
+      </c>
+    </row>
+    <row r="125" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A125">
+        <v>20</v>
+      </c>
+      <c r="B125">
+        <v>12</v>
+      </c>
+      <c r="C125">
+        <v>2</v>
+      </c>
+      <c r="D125">
         <f t="shared" si="28"/>
-        <v>235010.93054261635</v>
-      </c>
-      <c r="Q122">
-        <v>1247.3228025527501</v>
-      </c>
-      <c r="R122">
-        <v>16417.502561416801</v>
-      </c>
-      <c r="S122">
-        <v>469.07150175476602</v>
-      </c>
-      <c r="T122" s="6">
-        <v>0.46004655114715598</v>
-      </c>
-    </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A123">
-        <v>20</v>
-      </c>
-      <c r="B123">
-        <v>12</v>
-      </c>
-      <c r="C123">
-        <v>2</v>
-      </c>
-      <c r="D123">
-        <f t="shared" si="27"/>
         <v>114787.7594081375</v>
       </c>
-      <c r="E123">
+      <c r="E125">
         <v>282179.67123287602</v>
       </c>
-      <c r="F123">
+      <c r="F125">
         <v>0.83403396920434802</v>
       </c>
-      <c r="G123">
+      <c r="G125">
         <v>20436.472361711199</v>
       </c>
-      <c r="H123">
+      <c r="H125">
         <v>4946.5396722567002</v>
       </c>
-      <c r="I123">
+      <c r="I125">
         <v>2967.9237851293901</v>
       </c>
-      <c r="J123">
+      <c r="J125">
         <v>28350.9358190973</v>
       </c>
-      <c r="K123">
+      <c r="K125">
         <v>50843.184005923598</v>
       </c>
-      <c r="L123">
+      <c r="L125">
         <v>15303.798385783</v>
       </c>
-      <c r="M123">
+      <c r="M125">
         <v>19297.530489448302</v>
       </c>
-      <c r="N123">
+      <c r="N125">
         <v>992.31070788530405</v>
       </c>
-      <c r="O123">
-        <v>0</v>
-      </c>
-      <c r="P123">
-        <f t="shared" si="28"/>
+      <c r="O125">
+        <v>0</v>
+      </c>
+      <c r="P125">
+        <f t="shared" si="29"/>
         <v>235347.43122713402</v>
       </c>
-      <c r="Q123">
+      <c r="Q125">
         <v>1101.8639118583401</v>
       </c>
-      <c r="R123">
+      <c r="R125">
         <v>13.380488321454299</v>
       </c>
-      <c r="S123">
+      <c r="S125">
         <v>2.67609766429086</v>
       </c>
-      <c r="T123" s="6">
+      <c r="T125" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A64:C64"/>
     <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="A67:C67"/>
+    <mergeCell ref="A71:B71"/>
+    <mergeCell ref="A69:C69"/>
+    <mergeCell ref="A66:D66"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>